<commit_message>
Add Imitator, Trapper Plus, and Aurial roles
</commit_message>
<xml_diff>
--- a/Strings.xlsx
+++ b/Strings.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="3" r:id="Ra315dc42db004600"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other Text" sheetId="10" r:id="R6a0beecf73b147ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colors" sheetId="7" r:id="Rfcbca6ef2c1644ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Button Text" sheetId="8" r:id="R79ab9c48b5314d5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RoleInfo" sheetId="9" r:id="Rf319d6606c694eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Description" sheetId="11" r:id="Rf98df877173e4a85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="3" r:id="Rf852e54ab7d34179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other Text" sheetId="10" r:id="Rfc079b4b4a6348d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colors" sheetId="7" r:id="Rb5f356c2b5804109"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Button Text" sheetId="8" r:id="Rf347ec38db084b72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RoleInfo" sheetId="9" r:id="R0666374627f4470b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Description" sheetId="11" r:id="Rc8472b53626d4039"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12041,9 +12041,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Trapper</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">设陷师</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TrapperIntroDesc</x:t>
@@ -23797,37 +23794,279 @@
       </x:c>
     </x:row>
     <x:row r="881" ht="24.950000762939453" customHeight="1">
-      <x:c r="O881" s="2"/>
+      <x:c r="A881" t="str">
+        <x:v>trapperPlusMinDwellTime</x:v>
+      </x:c>
+      <x:c r="B881" t="str">
+        <x:v>Minimum Time in Trap</x:v>
+      </x:c>
+      <x:c r="C881"/>
+      <x:c r="D881"/>
+      <x:c r="E881"/>
+      <x:c r="F881"/>
+      <x:c r="G881"/>
+      <x:c r="H881"/>
+      <x:c r="I881"/>
+      <x:c r="J881"/>
+      <x:c r="K881"/>
+      <x:c r="L881"/>
+      <x:c r="M881"/>
+      <x:c r="N881"/>
+      <x:c r="O881" s="2" t="str">
+        <x:v>陷阱内最短停留时间</x:v>
+      </x:c>
+      <x:c r="P881"/>
+      <x:c r="Q881"/>
     </x:row>
     <x:row r="882" ht="24.950000762939453" customHeight="1">
-      <x:c r="O882" s="2"/>
+      <x:c r="A882" t="str">
+        <x:v>trapperPlusCooldown</x:v>
+      </x:c>
+      <x:c r="B882" t="str">
+        <x:v>Trap Placement Cooldown</x:v>
+      </x:c>
+      <x:c r="C882"/>
+      <x:c r="D882"/>
+      <x:c r="E882"/>
+      <x:c r="F882"/>
+      <x:c r="G882"/>
+      <x:c r="H882"/>
+      <x:c r="I882"/>
+      <x:c r="J882"/>
+      <x:c r="K882"/>
+      <x:c r="L882"/>
+      <x:c r="M882"/>
+      <x:c r="N882"/>
+      <x:c r="O882" s="2" t="str">
+        <x:v>放置陷阱冷却</x:v>
+      </x:c>
+      <x:c r="P882"/>
+      <x:c r="Q882"/>
     </x:row>
     <x:row r="883" ht="24.950000762939453" customHeight="1">
-      <x:c r="O883" s="2"/>
+      <x:c r="A883" t="str">
+        <x:v>trapperPlusRemoveTrapsEachRound</x:v>
+      </x:c>
+      <x:c r="B883" t="str">
+        <x:v>Remove Traps Each Round</x:v>
+      </x:c>
+      <x:c r="C883"/>
+      <x:c r="D883"/>
+      <x:c r="E883"/>
+      <x:c r="F883"/>
+      <x:c r="G883"/>
+      <x:c r="H883"/>
+      <x:c r="I883"/>
+      <x:c r="J883"/>
+      <x:c r="K883"/>
+      <x:c r="L883"/>
+      <x:c r="M883"/>
+      <x:c r="N883"/>
+      <x:c r="O883" s="2" t="str">
+        <x:v>每轮清除陷阱</x:v>
+      </x:c>
+      <x:c r="P883"/>
+      <x:c r="Q883"/>
     </x:row>
     <x:row r="884" ht="24.950000762939453" customHeight="1">
-      <x:c r="O884" s="2"/>
+      <x:c r="A884" t="str">
+        <x:v>trapperPlusMaxTraps</x:v>
+      </x:c>
+      <x:c r="B884" t="str">
+        <x:v>Maximum Number of Traps</x:v>
+      </x:c>
+      <x:c r="C884"/>
+      <x:c r="D884"/>
+      <x:c r="E884"/>
+      <x:c r="F884"/>
+      <x:c r="G884"/>
+      <x:c r="H884"/>
+      <x:c r="I884"/>
+      <x:c r="J884"/>
+      <x:c r="K884"/>
+      <x:c r="L884"/>
+      <x:c r="M884"/>
+      <x:c r="N884"/>
+      <x:c r="O884" s="2" t="str">
+        <x:v>最大陷阱数量</x:v>
+      </x:c>
+      <x:c r="P884"/>
+      <x:c r="Q884"/>
     </x:row>
     <x:row r="885" ht="24.950000762939453" customHeight="1">
-      <x:c r="O885" s="2"/>
+      <x:c r="A885" t="str">
+        <x:v>trapperPlusTrapSize</x:v>
+      </x:c>
+      <x:c r="B885" t="str">
+        <x:v>Trap Radius</x:v>
+      </x:c>
+      <x:c r="C885"/>
+      <x:c r="D885"/>
+      <x:c r="E885"/>
+      <x:c r="F885"/>
+      <x:c r="G885"/>
+      <x:c r="H885"/>
+      <x:c r="I885"/>
+      <x:c r="J885"/>
+      <x:c r="K885"/>
+      <x:c r="L885"/>
+      <x:c r="M885"/>
+      <x:c r="N885"/>
+      <x:c r="O885" s="2" t="str">
+        <x:v>陷阱半径</x:v>
+      </x:c>
+      <x:c r="P885"/>
+      <x:c r="Q885"/>
     </x:row>
     <x:row r="886" ht="24.950000762939453" customHeight="1">
-      <x:c r="O886" s="2"/>
+      <x:c r="A886" t="str">
+        <x:v>trapperPlusMinPlayersToReport</x:v>
+      </x:c>
+      <x:c r="B886" t="str">
+        <x:v>Minimum Players for Report</x:v>
+      </x:c>
+      <x:c r="C886"/>
+      <x:c r="D886"/>
+      <x:c r="E886"/>
+      <x:c r="F886"/>
+      <x:c r="G886"/>
+      <x:c r="H886"/>
+      <x:c r="I886"/>
+      <x:c r="J886"/>
+      <x:c r="K886"/>
+      <x:c r="L886"/>
+      <x:c r="M886"/>
+      <x:c r="N886"/>
+      <x:c r="O886" s="2" t="str">
+        <x:v>生成报告所需最少玩家数</x:v>
+      </x:c>
+      <x:c r="P886"/>
+      <x:c r="Q886"/>
     </x:row>
     <x:row r="887" ht="24.950000762939453" customHeight="1">
-      <x:c r="O887" s="2"/>
+      <x:c r="A887" t="str">
+        <x:v>aurialCooldown</x:v>
+      </x:c>
+      <x:c r="B887" t="str">
+        <x:v>Radiate Cooldown</x:v>
+      </x:c>
+      <x:c r="C887"/>
+      <x:c r="D887"/>
+      <x:c r="E887"/>
+      <x:c r="F887"/>
+      <x:c r="G887"/>
+      <x:c r="H887"/>
+      <x:c r="I887"/>
+      <x:c r="J887"/>
+      <x:c r="K887"/>
+      <x:c r="L887"/>
+      <x:c r="M887"/>
+      <x:c r="N887"/>
+      <x:c r="O887" s="2" t="str">
+        <x:v>辐射冷却</x:v>
+      </x:c>
+      <x:c r="P887"/>
+      <x:c r="Q887"/>
     </x:row>
     <x:row r="888" ht="24.950000762939453" customHeight="1">
-      <x:c r="O888" s="2"/>
+      <x:c r="A888" t="str">
+        <x:v>aurialRadius</x:v>
+      </x:c>
+      <x:c r="B888" t="str">
+        <x:v>Radiate Radius</x:v>
+      </x:c>
+      <x:c r="C888"/>
+      <x:c r="D888"/>
+      <x:c r="E888"/>
+      <x:c r="F888"/>
+      <x:c r="G888"/>
+      <x:c r="H888"/>
+      <x:c r="I888"/>
+      <x:c r="J888"/>
+      <x:c r="K888"/>
+      <x:c r="L888"/>
+      <x:c r="M888"/>
+      <x:c r="N888"/>
+      <x:c r="O888" s="2" t="str">
+        <x:v>辐射范围</x:v>
+      </x:c>
+      <x:c r="P888"/>
+      <x:c r="Q888"/>
     </x:row>
     <x:row r="889" ht="24.950000762939453" customHeight="1">
-      <x:c r="O889" s="2"/>
+      <x:c r="A889" t="str">
+        <x:v>aurialHitsToReveal</x:v>
+      </x:c>
+      <x:c r="B889" t="str">
+        <x:v>Hits Required to Reveal Faction</x:v>
+      </x:c>
+      <x:c r="C889"/>
+      <x:c r="D889"/>
+      <x:c r="E889"/>
+      <x:c r="F889"/>
+      <x:c r="G889"/>
+      <x:c r="H889"/>
+      <x:c r="I889"/>
+      <x:c r="J889"/>
+      <x:c r="K889"/>
+      <x:c r="L889"/>
+      <x:c r="M889"/>
+      <x:c r="N889"/>
+      <x:c r="O889" s="2" t="str">
+        <x:v>识别阵营所需命中次数</x:v>
+      </x:c>
+      <x:c r="P889"/>
+      <x:c r="Q889"/>
     </x:row>
     <x:row r="890" ht="24.950000762939453" customHeight="1">
-      <x:c r="O890" s="2"/>
+      <x:c r="A890" t="str">
+        <x:v>aurialVision</x:v>
+      </x:c>
+      <x:c r="B890" t="str">
+        <x:v>Aurial Vision</x:v>
+      </x:c>
+      <x:c r="C890"/>
+      <x:c r="D890"/>
+      <x:c r="E890"/>
+      <x:c r="F890"/>
+      <x:c r="G890"/>
+      <x:c r="H890"/>
+      <x:c r="I890"/>
+      <x:c r="J890"/>
+      <x:c r="K890"/>
+      <x:c r="L890"/>
+      <x:c r="M890"/>
+      <x:c r="N890"/>
+      <x:c r="O890" s="2" t="str">
+        <x:v>灵光师视野</x:v>
+      </x:c>
+      <x:c r="P890"/>
+      <x:c r="Q890"/>
     </x:row>
     <x:row r="891" ht="24.950000762939453" customHeight="1">
-      <x:c r="O891" s="2"/>
+      <x:c r="A891" t="str">
+        <x:v>aurialAffectedByVortox</x:v>
+      </x:c>
+      <x:c r="B891" t="str">
+        <x:v>Aurial Affected by Vortox</x:v>
+      </x:c>
+      <x:c r="C891"/>
+      <x:c r="D891"/>
+      <x:c r="E891"/>
+      <x:c r="F891"/>
+      <x:c r="G891"/>
+      <x:c r="H891"/>
+      <x:c r="I891"/>
+      <x:c r="J891"/>
+      <x:c r="K891"/>
+      <x:c r="L891"/>
+      <x:c r="M891"/>
+      <x:c r="N891"/>
+      <x:c r="O891" s="2" t="str">
+        <x:v>灵光师受迷乱漩涡影响</x:v>
+      </x:c>
+      <x:c r="P891"/>
+      <x:c r="Q891"/>
     </x:row>
     <x:row r="892" ht="24.950000762939453" customHeight="1">
       <x:c r="O892" s="2"/>
@@ -29795,6 +30034,206 @@
       <x:c r="O312" s="16" t="s">
         <x:v>2921</x:v>
       </x:c>
+    </x:row>
+    <x:row r="313">
+      <x:c r="A313" t="str">
+        <x:v>TrapperPlus.Report.NoPlayers</x:v>
+      </x:c>
+      <x:c r="B313" t="str">
+        <x:v>Trap Report: No players triggered your traps.</x:v>
+      </x:c>
+      <x:c r="C313"/>
+      <x:c r="D313"/>
+      <x:c r="E313"/>
+      <x:c r="F313"/>
+      <x:c r="G313"/>
+      <x:c r="H313"/>
+      <x:c r="I313"/>
+      <x:c r="J313"/>
+      <x:c r="K313"/>
+      <x:c r="L313"/>
+      <x:c r="M313"/>
+      <x:c r="N313"/>
+      <x:c r="O313" t="str">
+        <x:v>陷阱报告：没有玩家触发你的陷阱。</x:v>
+      </x:c>
+      <x:c r="P313"/>
+      <x:c r="Q313"/>
+    </x:row>
+    <x:row r="314">
+      <x:c r="A314" t="str">
+        <x:v>TrapperPlus.Report.NotEnoughPlayers</x:v>
+      </x:c>
+      <x:c r="B314" t="str">
+        <x:v>Trap Report: Not enough players triggered your traps.</x:v>
+      </x:c>
+      <x:c r="C314"/>
+      <x:c r="D314"/>
+      <x:c r="E314"/>
+      <x:c r="F314"/>
+      <x:c r="G314"/>
+      <x:c r="H314"/>
+      <x:c r="I314"/>
+      <x:c r="J314"/>
+      <x:c r="K314"/>
+      <x:c r="L314"/>
+      <x:c r="M314"/>
+      <x:c r="N314"/>
+      <x:c r="O314" t="str">
+        <x:v>陷阱报告：触发人数不足，无法生成职业列表。</x:v>
+      </x:c>
+      <x:c r="P314"/>
+      <x:c r="Q314"/>
+    </x:row>
+    <x:row r="315">
+      <x:c r="A315" t="str">
+        <x:v>TrapperPlus.Report.Roles</x:v>
+      </x:c>
+      <x:c r="B315" t="str">
+        <x:v>Trap Report: Roles detected: {0}</x:v>
+      </x:c>
+      <x:c r="C315"/>
+      <x:c r="D315"/>
+      <x:c r="E315"/>
+      <x:c r="F315"/>
+      <x:c r="G315"/>
+      <x:c r="H315"/>
+      <x:c r="I315"/>
+      <x:c r="J315"/>
+      <x:c r="K315"/>
+      <x:c r="L315"/>
+      <x:c r="M315"/>
+      <x:c r="N315"/>
+      <x:c r="O315" t="str">
+        <x:v>陷阱报告：检测到的职业：{0}。</x:v>
+      </x:c>
+      <x:c r="P315"/>
+      <x:c r="Q315"/>
+    </x:row>
+    <x:row r="316">
+      <x:c r="A316" t="str">
+        <x:v>Imitator.Selection.Selected</x:v>
+      </x:c>
+      <x:c r="B316" t="str">
+        <x:v>Selected {0} to imitate.</x:v>
+      </x:c>
+      <x:c r="C316"/>
+      <x:c r="D316"/>
+      <x:c r="E316"/>
+      <x:c r="F316"/>
+      <x:c r="G316"/>
+      <x:c r="H316"/>
+      <x:c r="I316"/>
+      <x:c r="J316"/>
+      <x:c r="K316"/>
+      <x:c r="L316"/>
+      <x:c r="M316"/>
+      <x:c r="N316"/>
+      <x:c r="O316" t="str">
+        <x:v>已选择效仿 {0}。</x:v>
+      </x:c>
+      <x:c r="P316"/>
+      <x:c r="Q316"/>
+    </x:row>
+    <x:row r="317">
+      <x:c r="A317" t="str">
+        <x:v>Imitator.Selection.Cleared</x:v>
+      </x:c>
+      <x:c r="B317" t="str">
+        <x:v>Imitation target cleared.</x:v>
+      </x:c>
+      <x:c r="C317"/>
+      <x:c r="D317"/>
+      <x:c r="E317"/>
+      <x:c r="F317"/>
+      <x:c r="G317"/>
+      <x:c r="H317"/>
+      <x:c r="I317"/>
+      <x:c r="J317"/>
+      <x:c r="K317"/>
+      <x:c r="L317"/>
+      <x:c r="M317"/>
+      <x:c r="N317"/>
+      <x:c r="O317" t="str">
+        <x:v>已取消效仿目标。</x:v>
+      </x:c>
+      <x:c r="P317"/>
+      <x:c r="Q317"/>
+    </x:row>
+    <x:row r="318">
+      <x:c r="A318" t="str">
+        <x:v>Imitator.Selection.Invalid</x:v>
+      </x:c>
+      <x:c r="B318" t="str">
+        <x:v>This player cannot be imitated.</x:v>
+      </x:c>
+      <x:c r="C318"/>
+      <x:c r="D318"/>
+      <x:c r="E318"/>
+      <x:c r="F318"/>
+      <x:c r="G318"/>
+      <x:c r="H318"/>
+      <x:c r="I318"/>
+      <x:c r="J318"/>
+      <x:c r="K318"/>
+      <x:c r="L318"/>
+      <x:c r="M318"/>
+      <x:c r="N318"/>
+      <x:c r="O318" t="str">
+        <x:v>无法效仿该玩家。</x:v>
+      </x:c>
+      <x:c r="P318"/>
+      <x:c r="Q318"/>
+    </x:row>
+    <x:row r="319">
+      <x:c r="A319" t="str">
+        <x:v>Aurial.RadiationProgress</x:v>
+      </x:c>
+      <x:c r="B319" t="str">
+        <x:v>Radiation: {0} ({1}/{2})</x:v>
+      </x:c>
+      <x:c r="C319"/>
+      <x:c r="D319"/>
+      <x:c r="E319"/>
+      <x:c r="F319"/>
+      <x:c r="G319"/>
+      <x:c r="H319"/>
+      <x:c r="I319"/>
+      <x:c r="J319"/>
+      <x:c r="K319"/>
+      <x:c r="L319"/>
+      <x:c r="M319"/>
+      <x:c r="N319"/>
+      <x:c r="O319" t="str">
+        <x:v>辐射进度：{0}（{1}/{2}）</x:v>
+      </x:c>
+      <x:c r="P319"/>
+      <x:c r="Q319"/>
+    </x:row>
+    <x:row r="320">
+      <x:c r="A320" t="str">
+        <x:v>Aurial.RadiationUnlocked</x:v>
+      </x:c>
+      <x:c r="B320" t="str">
+        <x:v>Faction revealed for {0} ({1}/{2}).</x:v>
+      </x:c>
+      <x:c r="C320"/>
+      <x:c r="D320"/>
+      <x:c r="E320"/>
+      <x:c r="F320"/>
+      <x:c r="G320"/>
+      <x:c r="H320"/>
+      <x:c r="I320"/>
+      <x:c r="J320"/>
+      <x:c r="K320"/>
+      <x:c r="L320"/>
+      <x:c r="M320"/>
+      <x:c r="N320"/>
+      <x:c r="O320" t="str">
+        <x:v>已解锁 {0} 的阵营信息（{1}/{2}）。</x:v>
+      </x:c>
+      <x:c r="P320"/>
+      <x:c r="Q320"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31652,6 +32091,60 @@
         <x:v>3349</x:v>
       </x:c>
     </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>trapperPlusPlaceTrapText</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>PLACE TRAP</x:v>
+      </x:c>
+      <x:c r="C115"/>
+      <x:c r="D115"/>
+      <x:c r="E115"/>
+      <x:c r="F115"/>
+      <x:c r="G115"/>
+      <x:c r="H115"/>
+      <x:c r="I115"/>
+      <x:c r="J115"/>
+      <x:c r="K115"/>
+      <x:c r="L115"/>
+      <x:c r="M115"/>
+      <x:c r="N115"/>
+      <x:c r="O115" t="str">
+        <x:v>放置陷阱</x:v>
+      </x:c>
+      <x:c r="P115"/>
+      <x:c r="Q115"/>
+      <x:c r="R115"/>
+      <x:c r="S115"/>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>aurialRadiateText</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>RADIATE</x:v>
+      </x:c>
+      <x:c r="C116"/>
+      <x:c r="D116"/>
+      <x:c r="E116"/>
+      <x:c r="F116"/>
+      <x:c r="G116"/>
+      <x:c r="H116"/>
+      <x:c r="I116"/>
+      <x:c r="J116"/>
+      <x:c r="K116"/>
+      <x:c r="L116"/>
+      <x:c r="M116"/>
+      <x:c r="N116"/>
+      <x:c r="O116" t="str">
+        <x:v>辐射</x:v>
+      </x:c>
+      <x:c r="P116"/>
+      <x:c r="Q116"/>
+      <x:c r="R116"/>
+      <x:c r="S116"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -34264,591 +34757,591 @@
       <x:c r="B310" s="4" t="s">
         <x:v>3951</x:v>
       </x:c>
-      <x:c r="O310" s="4" t="s">
-        <x:v>3952</x:v>
+      <x:c r="O310" s="4" t="str">
+        <x:v>设陷师</x:v>
       </x:c>
     </x:row>
     <x:row r="311">
       <x:c r="A311" s="4" t="s">
+        <x:v>3952</x:v>
+      </x:c>
+      <x:c r="B311" s="4" t="s">
         <x:v>3953</x:v>
       </x:c>
-      <x:c r="B311" s="4" t="s">
+      <x:c r="O311" s="4" t="s">
         <x:v>3954</x:v>
-      </x:c>
-      <x:c r="O311" s="4" t="s">
-        <x:v>3955</x:v>
       </x:c>
     </x:row>
     <x:row r="312">
       <x:c r="A312" s="4" t="s">
+        <x:v>3955</x:v>
+      </x:c>
+      <x:c r="B312" s="4" t="s">
         <x:v>3956</x:v>
       </x:c>
-      <x:c r="B312" s="4" t="s">
+      <x:c r="O312" s="4" t="s">
         <x:v>3957</x:v>
-      </x:c>
-      <x:c r="O312" s="4" t="s">
-        <x:v>3958</x:v>
       </x:c>
     </x:row>
     <x:row r="314">
       <x:c r="A314" s="4" t="s">
+        <x:v>3958</x:v>
+      </x:c>
+      <x:c r="B314" s="4" t="s">
+        <x:v>3958</x:v>
+      </x:c>
+      <x:c r="O314" s="4" t="s">
         <x:v>3959</x:v>
-      </x:c>
-      <x:c r="B314" s="4" t="s">
-        <x:v>3959</x:v>
-      </x:c>
-      <x:c r="O314" s="4" t="s">
-        <x:v>3960</x:v>
       </x:c>
     </x:row>
     <x:row r="315">
       <x:c r="A315" s="4" t="s">
+        <x:v>3960</x:v>
+      </x:c>
+      <x:c r="B315" s="4" t="s">
         <x:v>3961</x:v>
       </x:c>
-      <x:c r="B315" s="4" t="s">
+      <x:c r="O315" s="4" t="s">
         <x:v>3962</x:v>
-      </x:c>
-      <x:c r="O315" s="4" t="s">
-        <x:v>3963</x:v>
       </x:c>
     </x:row>
     <x:row r="316">
       <x:c r="A316" s="4" t="s">
+        <x:v>3963</x:v>
+      </x:c>
+      <x:c r="B316" s="4" t="s">
         <x:v>3964</x:v>
       </x:c>
-      <x:c r="B316" s="4" t="s">
+      <x:c r="O316" s="4" t="s">
         <x:v>3965</x:v>
-      </x:c>
-      <x:c r="O316" s="4" t="s">
-        <x:v>3966</x:v>
       </x:c>
     </x:row>
     <x:row r="318">
       <x:c r="A318" s="4" t="s">
+        <x:v>3966</x:v>
+      </x:c>
+      <x:c r="B318" s="4" t="s">
         <x:v>3967</x:v>
       </x:c>
-      <x:c r="B318" s="4" t="s">
+      <x:c r="O318" s="4" t="s">
         <x:v>3968</x:v>
-      </x:c>
-      <x:c r="O318" s="4" t="s">
-        <x:v>3969</x:v>
       </x:c>
     </x:row>
     <x:row r="319">
       <x:c r="A319" s="4" t="s">
+        <x:v>3969</x:v>
+      </x:c>
+      <x:c r="B319" s="4" t="s">
         <x:v>3970</x:v>
       </x:c>
-      <x:c r="B319" s="4" t="s">
+      <x:c r="O319" s="4" t="s">
         <x:v>3971</x:v>
-      </x:c>
-      <x:c r="O319" s="4" t="s">
-        <x:v>3972</x:v>
       </x:c>
     </x:row>
     <x:row r="320">
       <x:c r="A320" s="4" t="s">
+        <x:v>3972</x:v>
+      </x:c>
+      <x:c r="B320" s="4" t="s">
         <x:v>3973</x:v>
       </x:c>
-      <x:c r="B320" s="4" t="s">
+      <x:c r="O320" s="4" t="s">
         <x:v>3974</x:v>
-      </x:c>
-      <x:c r="O320" s="4" t="s">
-        <x:v>3975</x:v>
       </x:c>
     </x:row>
     <x:row r="322">
       <x:c r="A322" s="4" t="s">
+        <x:v>3975</x:v>
+      </x:c>
+      <x:c r="B322" s="14" t="s">
         <x:v>3976</x:v>
       </x:c>
-      <x:c r="B322" s="14" t="s">
+      <x:c r="O322" s="4" t="s">
         <x:v>3977</x:v>
-      </x:c>
-      <x:c r="O322" s="4" t="s">
-        <x:v>3978</x:v>
       </x:c>
     </x:row>
     <x:row r="323">
       <x:c r="A323" s="4" t="s">
+        <x:v>3978</x:v>
+      </x:c>
+      <x:c r="B323" s="4" t="s">
         <x:v>3979</x:v>
       </x:c>
-      <x:c r="B323" s="4" t="s">
+      <x:c r="O323" s="4" t="s">
         <x:v>3980</x:v>
-      </x:c>
-      <x:c r="O323" s="4" t="s">
-        <x:v>3981</x:v>
       </x:c>
     </x:row>
     <x:row r="324">
       <x:c r="A324" s="4" t="s">
+        <x:v>3981</x:v>
+      </x:c>
+      <x:c r="B324" s="4" t="s">
         <x:v>3982</x:v>
       </x:c>
-      <x:c r="B324" s="4" t="s">
+      <x:c r="O324" s="4" t="s">
         <x:v>3983</x:v>
-      </x:c>
-      <x:c r="O324" s="4" t="s">
-        <x:v>3984</x:v>
       </x:c>
     </x:row>
     <x:row r="326">
       <x:c r="A326" s="14" t="s">
+        <x:v>3984</x:v>
+      </x:c>
+      <x:c r="B326" s="14" t="s">
+        <x:v>3984</x:v>
+      </x:c>
+      <x:c r="O326" s="4" t="s">
         <x:v>3985</x:v>
-      </x:c>
-      <x:c r="B326" s="14" t="s">
-        <x:v>3985</x:v>
-      </x:c>
-      <x:c r="O326" s="4" t="s">
-        <x:v>3986</x:v>
       </x:c>
     </x:row>
     <x:row r="327">
       <x:c r="A327" s="4" t="s">
+        <x:v>3986</x:v>
+      </x:c>
+      <x:c r="B327" s="4" t="s">
         <x:v>3987</x:v>
       </x:c>
-      <x:c r="B327" s="4" t="s">
+      <x:c r="O327" s="4" t="s">
         <x:v>3988</x:v>
-      </x:c>
-      <x:c r="O327" s="4" t="s">
-        <x:v>3989</x:v>
       </x:c>
     </x:row>
     <x:row r="328">
       <x:c r="A328" s="4" t="s">
+        <x:v>3989</x:v>
+      </x:c>
+      <x:c r="B328" s="4" t="s">
         <x:v>3990</x:v>
       </x:c>
-      <x:c r="B328" s="4" t="s">
+      <x:c r="O328" s="4" t="s">
         <x:v>3991</x:v>
-      </x:c>
-      <x:c r="O328" s="4" t="s">
-        <x:v>3992</x:v>
       </x:c>
     </x:row>
     <x:row r="330">
       <x:c r="A330" s="4" t="s">
+        <x:v>3992</x:v>
+      </x:c>
+      <x:c r="B330" s="4" t="s">
+        <x:v>3992</x:v>
+      </x:c>
+      <x:c r="O330" s="4" t="s">
         <x:v>3993</x:v>
-      </x:c>
-      <x:c r="B330" s="4" t="s">
-        <x:v>3993</x:v>
-      </x:c>
-      <x:c r="O330" s="4" t="s">
-        <x:v>3994</x:v>
       </x:c>
     </x:row>
     <x:row r="331">
       <x:c r="A331" s="4" t="s">
+        <x:v>3994</x:v>
+      </x:c>
+      <x:c r="B331" s="4" t="s">
         <x:v>3995</x:v>
       </x:c>
-      <x:c r="B331" s="4" t="s">
+      <x:c r="O331" s="4" t="s">
         <x:v>3996</x:v>
-      </x:c>
-      <x:c r="O331" s="4" t="s">
-        <x:v>3997</x:v>
       </x:c>
     </x:row>
     <x:row r="332">
       <x:c r="A332" s="4" t="s">
+        <x:v>3997</x:v>
+      </x:c>
+      <x:c r="B332" s="4" t="s">
         <x:v>3998</x:v>
       </x:c>
-      <x:c r="B332" s="4" t="s">
+      <x:c r="O332" s="4" t="s">
         <x:v>3999</x:v>
-      </x:c>
-      <x:c r="O332" s="4" t="s">
-        <x:v>4000</x:v>
       </x:c>
     </x:row>
     <x:row r="334">
       <x:c r="A334" s="4" t="s">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="B334" s="4" t="s">
         <x:v>4001</x:v>
       </x:c>
-      <x:c r="B334" s="4" t="s">
+      <x:c r="O334" s="4" t="s">
         <x:v>4002</x:v>
-      </x:c>
-      <x:c r="O334" s="4" t="s">
-        <x:v>4003</x:v>
       </x:c>
     </x:row>
     <x:row r="335">
       <x:c r="A335" s="4" t="s">
+        <x:v>4003</x:v>
+      </x:c>
+      <x:c r="B335" s="4" t="s">
         <x:v>4004</x:v>
       </x:c>
-      <x:c r="B335" s="4" t="s">
+      <x:c r="O335" s="4" t="s">
         <x:v>4005</x:v>
-      </x:c>
-      <x:c r="O335" s="4" t="s">
-        <x:v>4006</x:v>
       </x:c>
     </x:row>
     <x:row r="336">
       <x:c r="A336" s="4" t="s">
+        <x:v>4006</x:v>
+      </x:c>
+      <x:c r="B336" s="4" t="s">
         <x:v>4007</x:v>
       </x:c>
-      <x:c r="B336" s="4" t="s">
+      <x:c r="O336" s="4" t="s">
         <x:v>4008</x:v>
-      </x:c>
-      <x:c r="O336" s="4" t="s">
-        <x:v>4009</x:v>
       </x:c>
     </x:row>
     <x:row r="338">
       <x:c r="A338" s="4" t="s">
+        <x:v>4009</x:v>
+      </x:c>
+      <x:c r="B338" s="4" t="s">
         <x:v>4010</x:v>
       </x:c>
-      <x:c r="B338" s="4" t="s">
+      <x:c r="O338" s="4" t="s">
         <x:v>4011</x:v>
-      </x:c>
-      <x:c r="O338" s="4" t="s">
-        <x:v>4012</x:v>
       </x:c>
     </x:row>
     <x:row r="339">
       <x:c r="A339" s="4" t="s">
+        <x:v>4012</x:v>
+      </x:c>
+      <x:c r="B339" s="4" t="s">
         <x:v>4013</x:v>
       </x:c>
-      <x:c r="B339" s="4" t="s">
+      <x:c r="O339" s="4" t="s">
         <x:v>4014</x:v>
-      </x:c>
-      <x:c r="O339" s="4" t="s">
-        <x:v>4015</x:v>
       </x:c>
     </x:row>
     <x:row r="340">
       <x:c r="A340" s="4" t="s">
+        <x:v>4015</x:v>
+      </x:c>
+      <x:c r="B340" s="4" t="s">
         <x:v>4016</x:v>
       </x:c>
-      <x:c r="B340" s="4" t="s">
+      <x:c r="O340" s="4" t="s">
         <x:v>4017</x:v>
-      </x:c>
-      <x:c r="O340" s="4" t="s">
-        <x:v>4018</x:v>
       </x:c>
     </x:row>
     <x:row r="342">
       <x:c r="A342" s="4" t="s">
+        <x:v>4018</x:v>
+      </x:c>
+      <x:c r="B342" s="4" t="s">
         <x:v>4019</x:v>
       </x:c>
-      <x:c r="B342" s="4" t="s">
+      <x:c r="O342" s="4" t="s">
         <x:v>4020</x:v>
-      </x:c>
-      <x:c r="O342" s="4" t="s">
-        <x:v>4021</x:v>
       </x:c>
     </x:row>
     <x:row r="343">
       <x:c r="A343" s="4" t="s">
+        <x:v>4021</x:v>
+      </x:c>
+      <x:c r="B343" s="4" t="s">
         <x:v>4022</x:v>
       </x:c>
-      <x:c r="B343" s="4" t="s">
+      <x:c r="O343" s="4" t="s">
         <x:v>4023</x:v>
-      </x:c>
-      <x:c r="O343" s="4" t="s">
-        <x:v>4024</x:v>
       </x:c>
     </x:row>
     <x:row r="344">
       <x:c r="A344" s="4" t="s">
+        <x:v>4024</x:v>
+      </x:c>
+      <x:c r="B344" s="4" t="s">
         <x:v>4025</x:v>
       </x:c>
-      <x:c r="B344" s="4" t="s">
+      <x:c r="O344" s="4" t="s">
         <x:v>4026</x:v>
-      </x:c>
-      <x:c r="O344" s="4" t="s">
-        <x:v>4027</x:v>
       </x:c>
     </x:row>
     <x:row r="346">
       <x:c r="A346" s="4" t="s">
+        <x:v>4027</x:v>
+      </x:c>
+      <x:c r="B346" s="4" t="s">
+        <x:v>4027</x:v>
+      </x:c>
+      <x:c r="O346" s="4" t="s">
         <x:v>4028</x:v>
-      </x:c>
-      <x:c r="B346" s="4" t="s">
-        <x:v>4028</x:v>
-      </x:c>
-      <x:c r="O346" s="4" t="s">
-        <x:v>4029</x:v>
       </x:c>
     </x:row>
     <x:row r="347">
       <x:c r="A347" s="4" t="s">
+        <x:v>4029</x:v>
+      </x:c>
+      <x:c r="B347" s="4" t="s">
         <x:v>4030</x:v>
       </x:c>
-      <x:c r="B347" s="4" t="s">
+      <x:c r="O347" s="4" t="s">
         <x:v>4031</x:v>
-      </x:c>
-      <x:c r="O347" s="4" t="s">
-        <x:v>4032</x:v>
       </x:c>
     </x:row>
     <x:row r="348">
       <x:c r="A348" s="4" t="s">
+        <x:v>4032</x:v>
+      </x:c>
+      <x:c r="B348" s="4" t="s">
         <x:v>4033</x:v>
       </x:c>
-      <x:c r="B348" s="4" t="s">
+      <x:c r="O348" s="4" t="s">
         <x:v>4034</x:v>
-      </x:c>
-      <x:c r="O348" s="4" t="s">
-        <x:v>4035</x:v>
       </x:c>
     </x:row>
     <x:row r="350">
       <x:c r="A350" s="4" t="s">
+        <x:v>4035</x:v>
+      </x:c>
+      <x:c r="B350" s="4" t="s">
         <x:v>4036</x:v>
       </x:c>
-      <x:c r="B350" s="4" t="s">
+      <x:c r="O350" s="4" t="s">
         <x:v>4037</x:v>
-      </x:c>
-      <x:c r="O350" s="4" t="s">
-        <x:v>4038</x:v>
       </x:c>
     </x:row>
     <x:row r="351">
       <x:c r="A351" s="4" t="s">
+        <x:v>4038</x:v>
+      </x:c>
+      <x:c r="B351" s="4" t="s">
         <x:v>4039</x:v>
       </x:c>
-      <x:c r="B351" s="4" t="s">
+      <x:c r="O351" s="4" t="s">
         <x:v>4040</x:v>
-      </x:c>
-      <x:c r="O351" s="4" t="s">
-        <x:v>4041</x:v>
       </x:c>
     </x:row>
     <x:row r="352">
       <x:c r="A352" s="4" t="s">
-        <x:v>4042</x:v>
+        <x:v>4041</x:v>
       </x:c>
       <x:c r="B352" s="4" t="s">
+        <x:v>4039</x:v>
+      </x:c>
+      <x:c r="O352" s="4" t="s">
         <x:v>4040</x:v>
-      </x:c>
-      <x:c r="O352" s="4" t="s">
-        <x:v>4041</x:v>
       </x:c>
     </x:row>
     <x:row r="354">
       <x:c r="A354" s="4" t="s">
+        <x:v>4042</x:v>
+      </x:c>
+      <x:c r="B354" s="4" t="s">
         <x:v>4043</x:v>
       </x:c>
-      <x:c r="B354" s="4" t="s">
+      <x:c r="O354" s="4" t="s">
         <x:v>4044</x:v>
-      </x:c>
-      <x:c r="O354" s="4" t="s">
-        <x:v>4045</x:v>
       </x:c>
     </x:row>
     <x:row r="355">
       <x:c r="A355" s="4" t="s">
+        <x:v>4045</x:v>
+      </x:c>
+      <x:c r="B355" s="4" t="s">
         <x:v>4046</x:v>
       </x:c>
-      <x:c r="B355" s="4" t="s">
+      <x:c r="O355" s="4" t="s">
         <x:v>4047</x:v>
-      </x:c>
-      <x:c r="O355" s="4" t="s">
-        <x:v>4048</x:v>
       </x:c>
     </x:row>
     <x:row r="356">
       <x:c r="A356" s="4" t="s">
+        <x:v>4048</x:v>
+      </x:c>
+      <x:c r="B356" s="4" t="s">
         <x:v>4049</x:v>
       </x:c>
-      <x:c r="B356" s="4" t="s">
+      <x:c r="O356" s="4" t="s">
         <x:v>4050</x:v>
-      </x:c>
-      <x:c r="O356" s="4" t="s">
-        <x:v>4051</x:v>
       </x:c>
     </x:row>
     <x:row r="358">
       <x:c r="A358" s="4" t="s">
+        <x:v>4051</x:v>
+      </x:c>
+      <x:c r="B358" s="4" t="s">
+        <x:v>4051</x:v>
+      </x:c>
+      <x:c r="O358" s="4" t="s">
         <x:v>4052</x:v>
-      </x:c>
-      <x:c r="B358" s="4" t="s">
-        <x:v>4052</x:v>
-      </x:c>
-      <x:c r="O358" s="4" t="s">
-        <x:v>4053</x:v>
       </x:c>
     </x:row>
     <x:row r="359">
       <x:c r="A359" s="4" t="s">
+        <x:v>4053</x:v>
+      </x:c>
+      <x:c r="B359" s="4" t="s">
         <x:v>4054</x:v>
       </x:c>
-      <x:c r="B359" s="4" t="s">
+      <x:c r="O359" s="4" t="s">
         <x:v>4055</x:v>
-      </x:c>
-      <x:c r="O359" s="4" t="s">
-        <x:v>4056</x:v>
       </x:c>
     </x:row>
     <x:row r="360">
       <x:c r="A360" s="4" t="s">
+        <x:v>4056</x:v>
+      </x:c>
+      <x:c r="B360" s="4" t="s">
         <x:v>4057</x:v>
       </x:c>
-      <x:c r="B360" s="4" t="s">
+      <x:c r="O360" s="4" t="s">
         <x:v>4058</x:v>
-      </x:c>
-      <x:c r="O360" s="4" t="s">
-        <x:v>4059</x:v>
       </x:c>
     </x:row>
     <x:row r="362">
       <x:c r="A362" s="4" t="s">
+        <x:v>4059</x:v>
+      </x:c>
+      <x:c r="B362" s="4" t="s">
+        <x:v>4059</x:v>
+      </x:c>
+      <x:c r="O362" s="4" t="s">
         <x:v>4060</x:v>
-      </x:c>
-      <x:c r="B362" s="4" t="s">
-        <x:v>4060</x:v>
-      </x:c>
-      <x:c r="O362" s="4" t="s">
-        <x:v>4061</x:v>
       </x:c>
     </x:row>
     <x:row r="363">
       <x:c r="A363" s="4" t="s">
+        <x:v>4061</x:v>
+      </x:c>
+      <x:c r="B363" s="4" t="s">
         <x:v>4062</x:v>
       </x:c>
-      <x:c r="B363" s="4" t="s">
+      <x:c r="O363" s="4" t="s">
         <x:v>4063</x:v>
-      </x:c>
-      <x:c r="O363" s="4" t="s">
-        <x:v>4064</x:v>
       </x:c>
     </x:row>
     <x:row r="364">
       <x:c r="A364" s="4" t="s">
+        <x:v>4064</x:v>
+      </x:c>
+      <x:c r="B364" s="4" t="s">
         <x:v>4065</x:v>
       </x:c>
-      <x:c r="B364" s="4" t="s">
+      <x:c r="O364" s="4" t="s">
         <x:v>4066</x:v>
-      </x:c>
-      <x:c r="O364" s="4" t="s">
-        <x:v>4067</x:v>
       </x:c>
     </x:row>
     <x:row r="366">
       <x:c r="A366" s="4" t="s">
+        <x:v>4067</x:v>
+      </x:c>
+      <x:c r="B366" s="4" t="s">
+        <x:v>4067</x:v>
+      </x:c>
+      <x:c r="O366" s="4" t="s">
         <x:v>4068</x:v>
-      </x:c>
-      <x:c r="B366" s="4" t="s">
-        <x:v>4068</x:v>
-      </x:c>
-      <x:c r="O366" s="4" t="s">
-        <x:v>4069</x:v>
       </x:c>
     </x:row>
     <x:row r="367">
       <x:c r="A367" s="4" t="s">
+        <x:v>4069</x:v>
+      </x:c>
+      <x:c r="B367" s="4" t="s">
         <x:v>4070</x:v>
       </x:c>
-      <x:c r="B367" s="4" t="s">
+      <x:c r="O367" s="4" t="s">
         <x:v>4071</x:v>
-      </x:c>
-      <x:c r="O367" s="4" t="s">
-        <x:v>4072</x:v>
       </x:c>
     </x:row>
     <x:row r="368">
       <x:c r="A368" s="4" t="s">
+        <x:v>4072</x:v>
+      </x:c>
+      <x:c r="B368" s="4" t="s">
         <x:v>4073</x:v>
       </x:c>
-      <x:c r="B368" s="4" t="s">
+      <x:c r="O368" s="4" t="s">
         <x:v>4074</x:v>
-      </x:c>
-      <x:c r="O368" s="4" t="s">
-        <x:v>4075</x:v>
       </x:c>
     </x:row>
     <x:row r="370">
       <x:c r="A370" s="4" t="s">
+        <x:v>4075</x:v>
+      </x:c>
+      <x:c r="B370" s="4" t="s">
+        <x:v>4075</x:v>
+      </x:c>
+      <x:c r="O370" s="4" t="s">
         <x:v>4076</x:v>
-      </x:c>
-      <x:c r="B370" s="4" t="s">
-        <x:v>4076</x:v>
-      </x:c>
-      <x:c r="O370" s="4" t="s">
-        <x:v>4077</x:v>
       </x:c>
     </x:row>
     <x:row r="371">
       <x:c r="A371" s="4" t="s">
+        <x:v>4077</x:v>
+      </x:c>
+      <x:c r="B371" s="4" t="s">
         <x:v>4078</x:v>
       </x:c>
-      <x:c r="B371" s="4" t="s">
+      <x:c r="O371" s="4" t="s">
         <x:v>4079</x:v>
-      </x:c>
-      <x:c r="O371" s="4" t="s">
-        <x:v>4080</x:v>
       </x:c>
     </x:row>
     <x:row r="372">
       <x:c r="A372" s="4" t="s">
+        <x:v>4080</x:v>
+      </x:c>
+      <x:c r="B372" s="4" t="s">
         <x:v>4081</x:v>
       </x:c>
-      <x:c r="B372" s="4" t="s">
+      <x:c r="O372" s="4" t="s">
         <x:v>4082</x:v>
-      </x:c>
-      <x:c r="O372" s="4" t="s">
-        <x:v>4083</x:v>
       </x:c>
     </x:row>
     <x:row r="374">
       <x:c r="A374" s="4" t="s">
+        <x:v>4083</x:v>
+      </x:c>
+      <x:c r="B374" s="4" t="s">
+        <x:v>4083</x:v>
+      </x:c>
+      <x:c r="O374" s="4" t="s">
         <x:v>4084</x:v>
-      </x:c>
-      <x:c r="B374" s="4" t="s">
-        <x:v>4084</x:v>
-      </x:c>
-      <x:c r="O374" s="4" t="s">
-        <x:v>4085</x:v>
       </x:c>
     </x:row>
     <x:row r="375">
       <x:c r="A375" s="4" t="s">
+        <x:v>4085</x:v>
+      </x:c>
+      <x:c r="B375" s="4" t="s">
         <x:v>4086</x:v>
       </x:c>
-      <x:c r="B375" s="4" t="s">
+      <x:c r="O375" s="4" t="s">
         <x:v>4087</x:v>
-      </x:c>
-      <x:c r="O375" s="4" t="s">
-        <x:v>4088</x:v>
       </x:c>
     </x:row>
     <x:row r="376">
       <x:c r="A376" s="4" t="s">
+        <x:v>4088</x:v>
+      </x:c>
+      <x:c r="B376" s="4" t="s">
         <x:v>4089</x:v>
       </x:c>
-      <x:c r="B376" s="4" t="s">
+      <x:c r="O376" s="4" t="s">
         <x:v>4090</x:v>
-      </x:c>
-      <x:c r="O376" s="4" t="s">
-        <x:v>4091</x:v>
       </x:c>
     </x:row>
     <x:row r="378">
       <x:c r="A378" s="4" t="s">
+        <x:v>4091</x:v>
+      </x:c>
+      <x:c r="B378" s="4" t="s">
+        <x:v>4091</x:v>
+      </x:c>
+      <x:c r="O378" s="4" t="s">
         <x:v>4092</x:v>
-      </x:c>
-      <x:c r="B378" s="4" t="s">
-        <x:v>4092</x:v>
-      </x:c>
-      <x:c r="O378" s="4" t="s">
-        <x:v>4093</x:v>
       </x:c>
     </x:row>
     <x:row r="379">
       <x:c r="A379" s="4" t="s">
+        <x:v>4093</x:v>
+      </x:c>
+      <x:c r="B379" s="4" t="s">
         <x:v>4094</x:v>
       </x:c>
-      <x:c r="B379" s="4" t="s">
+      <x:c r="O379" s="4" t="s">
         <x:v>4095</x:v>
-      </x:c>
-      <x:c r="O379" s="4" t="s">
-        <x:v>4096</x:v>
       </x:c>
     </x:row>
     <x:row r="380">
       <x:c r="A380" s="4" t="s">
+        <x:v>4096</x:v>
+      </x:c>
+      <x:c r="B380" s="4" t="s">
         <x:v>4097</x:v>
       </x:c>
-      <x:c r="B380" s="4" t="s">
+      <x:c r="O380" s="4" t="s">
         <x:v>4098</x:v>
-      </x:c>
-      <x:c r="O380" s="4" t="s">
-        <x:v>4099</x:v>
       </x:c>
     </x:row>
     <x:row r="382">
@@ -34864,585 +35357,585 @@
     </x:row>
     <x:row r="383">
       <x:c r="A383" s="4" t="s">
+        <x:v>4099</x:v>
+      </x:c>
+      <x:c r="B383" s="4" t="s">
         <x:v>4100</x:v>
       </x:c>
-      <x:c r="B383" s="4" t="s">
+      <x:c r="O383" s="4" t="s">
         <x:v>4101</x:v>
-      </x:c>
-      <x:c r="O383" s="4" t="s">
-        <x:v>4102</x:v>
       </x:c>
     </x:row>
     <x:row r="384">
       <x:c r="A384" s="4" t="s">
-        <x:v>4103</x:v>
+        <x:v>4102</x:v>
       </x:c>
       <x:c r="B384" s="4" t="s">
+        <x:v>4100</x:v>
+      </x:c>
+      <x:c r="O384" s="4" t="s">
         <x:v>4101</x:v>
-      </x:c>
-      <x:c r="O384" s="4" t="s">
-        <x:v>4102</x:v>
       </x:c>
     </x:row>
     <x:row r="386">
       <x:c r="A386" s="4" t="s">
+        <x:v>4103</x:v>
+      </x:c>
+      <x:c r="B386" s="4" t="s">
+        <x:v>4103</x:v>
+      </x:c>
+      <x:c r="O386" s="4" t="s">
         <x:v>4104</x:v>
-      </x:c>
-      <x:c r="B386" s="4" t="s">
-        <x:v>4104</x:v>
-      </x:c>
-      <x:c r="O386" s="4" t="s">
-        <x:v>4105</x:v>
       </x:c>
     </x:row>
     <x:row r="387">
       <x:c r="A387" s="4" t="s">
+        <x:v>4105</x:v>
+      </x:c>
+      <x:c r="B387" s="4" t="s">
         <x:v>4106</x:v>
       </x:c>
-      <x:c r="B387" s="4" t="s">
+      <x:c r="O387" s="4" t="s">
         <x:v>4107</x:v>
-      </x:c>
-      <x:c r="O387" s="4" t="s">
-        <x:v>4108</x:v>
       </x:c>
     </x:row>
     <x:row r="388">
       <x:c r="A388" s="4" t="s">
+        <x:v>4108</x:v>
+      </x:c>
+      <x:c r="B388" s="4" t="s">
         <x:v>4109</x:v>
       </x:c>
-      <x:c r="B388" s="4" t="s">
+      <x:c r="O388" s="4" t="s">
         <x:v>4110</x:v>
-      </x:c>
-      <x:c r="O388" s="4" t="s">
-        <x:v>4111</x:v>
       </x:c>
     </x:row>
     <x:row r="390">
       <x:c r="A390" s="4" t="s">
+        <x:v>4111</x:v>
+      </x:c>
+      <x:c r="B390" s="4" t="s">
+        <x:v>4111</x:v>
+      </x:c>
+      <x:c r="O390" s="4" t="s">
         <x:v>4112</x:v>
-      </x:c>
-      <x:c r="B390" s="4" t="s">
-        <x:v>4112</x:v>
-      </x:c>
-      <x:c r="O390" s="4" t="s">
-        <x:v>4113</x:v>
       </x:c>
     </x:row>
     <x:row r="391">
       <x:c r="A391" s="4" t="s">
+        <x:v>4113</x:v>
+      </x:c>
+      <x:c r="B391" s="4" t="s">
         <x:v>4114</x:v>
       </x:c>
-      <x:c r="B391" s="4" t="s">
+      <x:c r="O391" s="4" t="s">
         <x:v>4115</x:v>
-      </x:c>
-      <x:c r="O391" s="4" t="s">
-        <x:v>4116</x:v>
       </x:c>
     </x:row>
     <x:row r="392">
       <x:c r="A392" s="4" t="s">
+        <x:v>4116</x:v>
+      </x:c>
+      <x:c r="B392" s="4" t="s">
         <x:v>4117</x:v>
       </x:c>
-      <x:c r="B392" s="4" t="s">
+      <x:c r="O392" s="4" t="s">
         <x:v>4118</x:v>
-      </x:c>
-      <x:c r="O392" s="4" t="s">
-        <x:v>4119</x:v>
       </x:c>
     </x:row>
     <x:row r="394">
       <x:c r="A394" s="4" t="s">
+        <x:v>4119</x:v>
+      </x:c>
+      <x:c r="B394" s="4" t="s">
         <x:v>4120</x:v>
       </x:c>
-      <x:c r="B394" s="4" t="s">
-        <x:v>4121</x:v>
-      </x:c>
       <x:c r="O394" s="4" t="s">
-        <x:v>4121</x:v>
+        <x:v>4120</x:v>
       </x:c>
     </x:row>
     <x:row r="395">
       <x:c r="A395" s="4" t="s">
+        <x:v>4121</x:v>
+      </x:c>
+      <x:c r="B395" s="4" t="s">
         <x:v>4122</x:v>
       </x:c>
-      <x:c r="B395" s="4" t="s">
+      <x:c r="O395" s="4" t="s">
         <x:v>4123</x:v>
-      </x:c>
-      <x:c r="O395" s="4" t="s">
-        <x:v>4124</x:v>
       </x:c>
     </x:row>
     <x:row r="396">
       <x:c r="A396" s="4" t="s">
+        <x:v>4124</x:v>
+      </x:c>
+      <x:c r="B396" s="4" t="s">
         <x:v>4125</x:v>
       </x:c>
-      <x:c r="B396" s="4" t="s">
+      <x:c r="O396" s="4" t="s">
         <x:v>4126</x:v>
-      </x:c>
-      <x:c r="O396" s="4" t="s">
-        <x:v>4127</x:v>
       </x:c>
     </x:row>
     <x:row r="398">
       <x:c r="A398" s="4" t="s">
+        <x:v>4127</x:v>
+      </x:c>
+      <x:c r="B398" s="4" t="s">
+        <x:v>4127</x:v>
+      </x:c>
+      <x:c r="O398" s="4" t="s">
         <x:v>4128</x:v>
-      </x:c>
-      <x:c r="B398" s="4" t="s">
-        <x:v>4128</x:v>
-      </x:c>
-      <x:c r="O398" s="4" t="s">
-        <x:v>4129</x:v>
       </x:c>
     </x:row>
     <x:row r="399">
       <x:c r="A399" s="4" t="s">
+        <x:v>4129</x:v>
+      </x:c>
+      <x:c r="B399" s="4" t="s">
         <x:v>4130</x:v>
       </x:c>
-      <x:c r="B399" s="4" t="s">
+      <x:c r="O399" s="4" t="s">
         <x:v>4131</x:v>
-      </x:c>
-      <x:c r="O399" s="4" t="s">
-        <x:v>4132</x:v>
       </x:c>
     </x:row>
     <x:row r="400">
       <x:c r="A400" s="4" t="s">
+        <x:v>4132</x:v>
+      </x:c>
+      <x:c r="B400" s="4" t="s">
         <x:v>4133</x:v>
       </x:c>
-      <x:c r="B400" s="4" t="s">
+      <x:c r="O400" s="4" t="s">
         <x:v>4134</x:v>
-      </x:c>
-      <x:c r="O400" s="4" t="s">
-        <x:v>4135</x:v>
       </x:c>
     </x:row>
     <x:row r="402">
       <x:c r="A402" s="4" t="s">
+        <x:v>4135</x:v>
+      </x:c>
+      <x:c r="B402" s="4" t="s">
         <x:v>4136</x:v>
       </x:c>
-      <x:c r="B402" s="4" t="s">
+      <x:c r="O402" s="4" t="s">
         <x:v>4137</x:v>
-      </x:c>
-      <x:c r="O402" s="4" t="s">
-        <x:v>4138</x:v>
       </x:c>
     </x:row>
     <x:row r="403">
       <x:c r="A403" s="4" t="s">
+        <x:v>4138</x:v>
+      </x:c>
+      <x:c r="B403" s="4" t="s">
         <x:v>4139</x:v>
       </x:c>
-      <x:c r="B403" s="4" t="s">
+      <x:c r="O403" s="4" t="s">
         <x:v>4140</x:v>
-      </x:c>
-      <x:c r="O403" s="4" t="s">
-        <x:v>4141</x:v>
       </x:c>
     </x:row>
     <x:row r="404">
       <x:c r="A404" s="4" t="s">
+        <x:v>4141</x:v>
+      </x:c>
+      <x:c r="B404" s="4" t="s">
         <x:v>4142</x:v>
       </x:c>
-      <x:c r="B404" s="4" t="s">
+      <x:c r="O404" s="4" t="s">
         <x:v>4143</x:v>
-      </x:c>
-      <x:c r="O404" s="4" t="s">
-        <x:v>4144</x:v>
       </x:c>
     </x:row>
     <x:row r="406">
       <x:c r="A406" s="4" t="s">
+        <x:v>4144</x:v>
+      </x:c>
+      <x:c r="B406" s="4" t="s">
         <x:v>4145</x:v>
       </x:c>
-      <x:c r="B406" s="4" t="s">
+      <x:c r="O406" s="4" t="s">
         <x:v>4146</x:v>
-      </x:c>
-      <x:c r="O406" s="4" t="s">
-        <x:v>4147</x:v>
       </x:c>
     </x:row>
     <x:row r="407">
       <x:c r="A407" s="4" t="s">
+        <x:v>4147</x:v>
+      </x:c>
+      <x:c r="B407" s="4" t="s">
         <x:v>4148</x:v>
       </x:c>
-      <x:c r="B407" s="4" t="s">
+      <x:c r="O407" s="4" t="s">
         <x:v>4149</x:v>
-      </x:c>
-      <x:c r="O407" s="4" t="s">
-        <x:v>4150</x:v>
       </x:c>
     </x:row>
     <x:row r="408">
       <x:c r="A408" s="4" t="s">
+        <x:v>4150</x:v>
+      </x:c>
+      <x:c r="B408" s="4" t="s">
         <x:v>4151</x:v>
       </x:c>
-      <x:c r="B408" s="4" t="s">
+      <x:c r="O408" s="4" t="s">
         <x:v>4152</x:v>
-      </x:c>
-      <x:c r="O408" s="4" t="s">
-        <x:v>4153</x:v>
       </x:c>
     </x:row>
     <x:row r="410">
       <x:c r="A410" s="4" t="s">
+        <x:v>4153</x:v>
+      </x:c>
+      <x:c r="B410" s="4" t="s">
         <x:v>4154</x:v>
       </x:c>
-      <x:c r="B410" s="4" t="s">
+      <x:c r="O410" s="4" t="s">
         <x:v>4155</x:v>
-      </x:c>
-      <x:c r="O410" s="4" t="s">
-        <x:v>4156</x:v>
       </x:c>
     </x:row>
     <x:row r="411">
       <x:c r="A411" s="4" t="s">
+        <x:v>4156</x:v>
+      </x:c>
+      <x:c r="B411" s="4" t="s">
         <x:v>4157</x:v>
       </x:c>
-      <x:c r="B411" s="4" t="s">
+      <x:c r="O411" s="4" t="s">
         <x:v>4158</x:v>
-      </x:c>
-      <x:c r="O411" s="4" t="s">
-        <x:v>4159</x:v>
       </x:c>
     </x:row>
     <x:row r="412">
       <x:c r="A412" s="4" t="s">
+        <x:v>4159</x:v>
+      </x:c>
+      <x:c r="B412" s="4" t="s">
         <x:v>4160</x:v>
       </x:c>
-      <x:c r="B412" s="4" t="s">
+      <x:c r="O412" s="4" t="s">
         <x:v>4161</x:v>
-      </x:c>
-      <x:c r="O412" s="4" t="s">
-        <x:v>4162</x:v>
       </x:c>
     </x:row>
     <x:row r="414">
       <x:c r="A414" s="4" t="s">
+        <x:v>4162</x:v>
+      </x:c>
+      <x:c r="B414" s="4" t="s">
+        <x:v>4162</x:v>
+      </x:c>
+      <x:c r="O414" s="4" t="s">
         <x:v>4163</x:v>
-      </x:c>
-      <x:c r="B414" s="4" t="s">
-        <x:v>4163</x:v>
-      </x:c>
-      <x:c r="O414" s="4" t="s">
-        <x:v>4164</x:v>
       </x:c>
     </x:row>
     <x:row r="415">
       <x:c r="A415" s="4" t="s">
+        <x:v>4164</x:v>
+      </x:c>
+      <x:c r="B415" s="4" t="s">
         <x:v>4165</x:v>
       </x:c>
-      <x:c r="B415" s="4" t="s">
+      <x:c r="O415" s="4" t="s">
         <x:v>4166</x:v>
-      </x:c>
-      <x:c r="O415" s="4" t="s">
-        <x:v>4167</x:v>
       </x:c>
     </x:row>
     <x:row r="416">
       <x:c r="A416" s="4" t="s">
+        <x:v>4167</x:v>
+      </x:c>
+      <x:c r="B416" s="4" t="s">
         <x:v>4168</x:v>
       </x:c>
-      <x:c r="B416" s="4" t="s">
+      <x:c r="O416" s="4" t="s">
         <x:v>4169</x:v>
-      </x:c>
-      <x:c r="O416" s="4" t="s">
-        <x:v>4170</x:v>
       </x:c>
     </x:row>
     <x:row r="418">
       <x:c r="A418" s="4" t="s">
+        <x:v>4170</x:v>
+      </x:c>
+      <x:c r="B418" s="4" t="s">
+        <x:v>4170</x:v>
+      </x:c>
+      <x:c r="O418" s="4" t="s">
         <x:v>4171</x:v>
-      </x:c>
-      <x:c r="B418" s="4" t="s">
-        <x:v>4171</x:v>
-      </x:c>
-      <x:c r="O418" s="4" t="s">
-        <x:v>4172</x:v>
       </x:c>
     </x:row>
     <x:row r="419">
       <x:c r="A419" s="4" t="s">
+        <x:v>4172</x:v>
+      </x:c>
+      <x:c r="B419" s="4" t="s">
         <x:v>4173</x:v>
       </x:c>
-      <x:c r="B419" s="4" t="s">
+      <x:c r="O419" s="4" t="s">
         <x:v>4174</x:v>
-      </x:c>
-      <x:c r="O419" s="4" t="s">
-        <x:v>4175</x:v>
       </x:c>
     </x:row>
     <x:row r="420">
       <x:c r="A420" s="4" t="s">
+        <x:v>4175</x:v>
+      </x:c>
+      <x:c r="B420" s="4" t="s">
         <x:v>4176</x:v>
       </x:c>
-      <x:c r="B420" s="4" t="s">
+      <x:c r="O420" s="4" t="s">
         <x:v>4177</x:v>
-      </x:c>
-      <x:c r="O420" s="4" t="s">
-        <x:v>4178</x:v>
       </x:c>
     </x:row>
     <x:row r="422">
       <x:c r="A422" s="4" t="s">
+        <x:v>4178</x:v>
+      </x:c>
+      <x:c r="B422" s="4" t="s">
+        <x:v>4178</x:v>
+      </x:c>
+      <x:c r="O422" s="4" t="s">
         <x:v>4179</x:v>
-      </x:c>
-      <x:c r="B422" s="4" t="s">
-        <x:v>4179</x:v>
-      </x:c>
-      <x:c r="O422" s="4" t="s">
-        <x:v>4180</x:v>
       </x:c>
     </x:row>
     <x:row r="423">
       <x:c r="A423" s="4" t="s">
+        <x:v>4180</x:v>
+      </x:c>
+      <x:c r="B423" s="4" t="s">
         <x:v>4181</x:v>
       </x:c>
-      <x:c r="B423" s="4" t="s">
+      <x:c r="O423" s="4" t="s">
         <x:v>4182</x:v>
-      </x:c>
-      <x:c r="O423" s="4" t="s">
-        <x:v>4183</x:v>
       </x:c>
     </x:row>
     <x:row r="424">
       <x:c r="A424" s="4" t="s">
+        <x:v>4183</x:v>
+      </x:c>
+      <x:c r="B424" s="4" t="s">
         <x:v>4184</x:v>
       </x:c>
-      <x:c r="B424" s="4" t="s">
+      <x:c r="O424" s="4" t="s">
         <x:v>4185</x:v>
-      </x:c>
-      <x:c r="O424" s="4" t="s">
-        <x:v>4186</x:v>
       </x:c>
     </x:row>
     <x:row r="426">
       <x:c r="A426" s="4" t="s">
+        <x:v>4186</x:v>
+      </x:c>
+      <x:c r="B426" s="4" t="s">
+        <x:v>4186</x:v>
+      </x:c>
+      <x:c r="O426" s="4" t="s">
         <x:v>4187</x:v>
-      </x:c>
-      <x:c r="B426" s="4" t="s">
-        <x:v>4187</x:v>
-      </x:c>
-      <x:c r="O426" s="4" t="s">
-        <x:v>4188</x:v>
       </x:c>
     </x:row>
     <x:row r="427">
       <x:c r="A427" s="4" t="s">
+        <x:v>4188</x:v>
+      </x:c>
+      <x:c r="B427" s="5" t="s">
         <x:v>4189</x:v>
       </x:c>
-      <x:c r="B427" s="5" t="s">
+      <x:c r="O427" s="4" t="s">
         <x:v>4190</x:v>
-      </x:c>
-      <x:c r="O427" s="4" t="s">
-        <x:v>4191</x:v>
       </x:c>
     </x:row>
     <x:row r="428">
       <x:c r="A428" s="4" t="s">
+        <x:v>4191</x:v>
+      </x:c>
+      <x:c r="B428" s="4" t="s">
         <x:v>4192</x:v>
       </x:c>
-      <x:c r="B428" s="4" t="s">
+      <x:c r="O428" s="4" t="s">
         <x:v>4193</x:v>
-      </x:c>
-      <x:c r="O428" s="4" t="s">
-        <x:v>4194</x:v>
       </x:c>
     </x:row>
     <x:row r="430">
       <x:c r="A430" s="4" t="s">
+        <x:v>4194</x:v>
+      </x:c>
+      <x:c r="B430" s="4" t="s">
         <x:v>4195</x:v>
       </x:c>
-      <x:c r="B430" s="4" t="s">
+      <x:c r="O430" s="4" t="s">
         <x:v>4196</x:v>
-      </x:c>
-      <x:c r="O430" s="4" t="s">
-        <x:v>4197</x:v>
       </x:c>
     </x:row>
     <x:row r="431">
       <x:c r="A431" s="4" t="s">
+        <x:v>4197</x:v>
+      </x:c>
+      <x:c r="B431" s="4" t="s">
         <x:v>4198</x:v>
       </x:c>
-      <x:c r="B431" s="4" t="s">
+      <x:c r="O431" s="4" t="s">
         <x:v>4199</x:v>
-      </x:c>
-      <x:c r="O431" s="4" t="s">
-        <x:v>4200</x:v>
       </x:c>
     </x:row>
     <x:row r="432">
       <x:c r="A432" s="4" t="s">
-        <x:v>4201</x:v>
+        <x:v>4200</x:v>
       </x:c>
       <x:c r="B432" s="4" t="s">
+        <x:v>4198</x:v>
+      </x:c>
+      <x:c r="O432" s="4" t="s">
         <x:v>4199</x:v>
-      </x:c>
-      <x:c r="O432" s="4" t="s">
-        <x:v>4200</x:v>
       </x:c>
     </x:row>
     <x:row r="434">
       <x:c r="A434" s="4" t="s">
+        <x:v>4201</x:v>
+      </x:c>
+      <x:c r="B434" s="4" t="s">
+        <x:v>4201</x:v>
+      </x:c>
+      <x:c r="O434" s="4" t="s">
         <x:v>4202</x:v>
-      </x:c>
-      <x:c r="B434" s="4" t="s">
-        <x:v>4202</x:v>
-      </x:c>
-      <x:c r="O434" s="4" t="s">
-        <x:v>4203</x:v>
       </x:c>
     </x:row>
     <x:row r="435">
       <x:c r="A435" s="4" t="s">
+        <x:v>4203</x:v>
+      </x:c>
+      <x:c r="B435" s="4" t="s">
         <x:v>4204</x:v>
       </x:c>
-      <x:c r="B435" s="4" t="s">
+      <x:c r="O435" s="4" t="s">
         <x:v>4205</x:v>
-      </x:c>
-      <x:c r="O435" s="4" t="s">
-        <x:v>4206</x:v>
       </x:c>
     </x:row>
     <x:row r="436">
       <x:c r="A436" s="4" t="s">
+        <x:v>4206</x:v>
+      </x:c>
+      <x:c r="B436" s="4" t="s">
         <x:v>4207</x:v>
       </x:c>
-      <x:c r="B436" s="4" t="s">
+      <x:c r="O436" s="4" t="s">
         <x:v>4208</x:v>
-      </x:c>
-      <x:c r="O436" s="4" t="s">
-        <x:v>4209</x:v>
       </x:c>
     </x:row>
     <x:row r="438">
       <x:c r="A438" s="4" t="s">
+        <x:v>4209</x:v>
+      </x:c>
+      <x:c r="B438" s="4" t="s">
+        <x:v>4209</x:v>
+      </x:c>
+      <x:c r="O438" s="4" t="s">
         <x:v>4210</x:v>
-      </x:c>
-      <x:c r="B438" s="4" t="s">
-        <x:v>4210</x:v>
-      </x:c>
-      <x:c r="O438" s="4" t="s">
-        <x:v>4211</x:v>
       </x:c>
     </x:row>
     <x:row r="439">
       <x:c r="A439" s="4" t="s">
+        <x:v>4211</x:v>
+      </x:c>
+      <x:c r="B439" s="4" t="s">
         <x:v>4212</x:v>
       </x:c>
-      <x:c r="B439" s="4" t="s">
+      <x:c r="O439" s="4" t="s">
         <x:v>4213</x:v>
-      </x:c>
-      <x:c r="O439" s="4" t="s">
-        <x:v>4214</x:v>
       </x:c>
     </x:row>
     <x:row r="440">
       <x:c r="A440" s="4" t="s">
+        <x:v>4214</x:v>
+      </x:c>
+      <x:c r="B440" s="4" t="s">
         <x:v>4215</x:v>
       </x:c>
-      <x:c r="B440" s="4" t="s">
+      <x:c r="O440" s="4" t="s">
         <x:v>4216</x:v>
-      </x:c>
-      <x:c r="O440" s="4" t="s">
-        <x:v>4217</x:v>
       </x:c>
     </x:row>
     <x:row r="442">
       <x:c r="A442" s="4" t="s">
+        <x:v>4217</x:v>
+      </x:c>
+      <x:c r="B442" s="4" t="s">
         <x:v>4218</x:v>
       </x:c>
-      <x:c r="B442" s="4" t="s">
+      <x:c r="O442" s="4" t="s">
         <x:v>4219</x:v>
-      </x:c>
-      <x:c r="O442" s="4" t="s">
-        <x:v>4220</x:v>
       </x:c>
     </x:row>
     <x:row r="443">
       <x:c r="A443" s="4" t="s">
+        <x:v>4220</x:v>
+      </x:c>
+      <x:c r="B443" s="4" t="s">
         <x:v>4221</x:v>
       </x:c>
-      <x:c r="B443" s="4" t="s">
+      <x:c r="O443" s="4" t="s">
         <x:v>4222</x:v>
-      </x:c>
-      <x:c r="O443" s="4" t="s">
-        <x:v>4223</x:v>
       </x:c>
     </x:row>
     <x:row r="444">
       <x:c r="A444" s="4" t="s">
-        <x:v>4224</x:v>
+        <x:v>4223</x:v>
       </x:c>
       <x:c r="B444" s="4" t="s">
+        <x:v>4221</x:v>
+      </x:c>
+      <x:c r="O444" s="4" t="s">
         <x:v>4222</x:v>
-      </x:c>
-      <x:c r="O444" s="4" t="s">
-        <x:v>4223</x:v>
       </x:c>
     </x:row>
     <x:row r="446">
       <x:c r="A446" s="4" t="s">
+        <x:v>4224</x:v>
+      </x:c>
+      <x:c r="B446" s="4" t="s">
+        <x:v>4224</x:v>
+      </x:c>
+      <x:c r="O446" s="4" t="s">
         <x:v>4225</x:v>
-      </x:c>
-      <x:c r="B446" s="4" t="s">
-        <x:v>4225</x:v>
-      </x:c>
-      <x:c r="O446" s="4" t="s">
-        <x:v>4226</x:v>
       </x:c>
     </x:row>
     <x:row r="447">
       <x:c r="A447" s="4" t="s">
+        <x:v>4226</x:v>
+      </x:c>
+      <x:c r="B447" s="4" t="s">
         <x:v>4227</x:v>
       </x:c>
-      <x:c r="B447" s="4" t="s">
+      <x:c r="O447" s="4" t="s">
         <x:v>4228</x:v>
-      </x:c>
-      <x:c r="O447" s="4" t="s">
-        <x:v>4229</x:v>
       </x:c>
     </x:row>
     <x:row r="448">
       <x:c r="A448" s="4" t="s">
-        <x:v>4230</x:v>
+        <x:v>4229</x:v>
       </x:c>
       <x:c r="B448" s="4" t="s">
+        <x:v>4227</x:v>
+      </x:c>
+      <x:c r="O448" s="4" t="s">
         <x:v>4228</x:v>
-      </x:c>
-      <x:c r="O448" s="4" t="s">
-        <x:v>4229</x:v>
       </x:c>
     </x:row>
     <x:row r="450">
       <x:c r="A450" s="4" t="s">
+        <x:v>4230</x:v>
+      </x:c>
+      <x:c r="B450" s="4" t="s">
+        <x:v>4230</x:v>
+      </x:c>
+      <x:c r="O450" s="4" t="s">
         <x:v>4231</x:v>
-      </x:c>
-      <x:c r="B450" s="4" t="s">
-        <x:v>4231</x:v>
-      </x:c>
-      <x:c r="O450" s="4" t="s">
-        <x:v>4232</x:v>
       </x:c>
     </x:row>
     <x:row r="451">
       <x:c r="A451" s="4" t="s">
+        <x:v>4232</x:v>
+      </x:c>
+      <x:c r="B451" s="4" t="s">
         <x:v>4233</x:v>
       </x:c>
-      <x:c r="B451" s="4" t="s">
+      <x:c r="O451" s="4" t="s">
         <x:v>4234</x:v>
-      </x:c>
-      <x:c r="O451" s="4" t="s">
-        <x:v>4235</x:v>
       </x:c>
     </x:row>
     <x:row r="452">
       <x:c r="A452" s="4" t="s">
-        <x:v>4236</x:v>
+        <x:v>4235</x:v>
       </x:c>
       <x:c r="B452" s="4" t="s">
+        <x:v>4233</x:v>
+      </x:c>
+      <x:c r="O452" s="4" t="s">
         <x:v>4234</x:v>
-      </x:c>
-      <x:c r="O452" s="4" t="s">
-        <x:v>4235</x:v>
       </x:c>
     </x:row>
     <x:row r="454">
@@ -35450,7 +35943,7 @@
         <x:v>2226</x:v>
       </x:c>
       <x:c r="B454" s="4" t="s">
-        <x:v>4237</x:v>
+        <x:v>4236</x:v>
       </x:c>
       <x:c r="O454" s="4" t="s">
         <x:v>2227</x:v>
@@ -35458,10 +35951,10 @@
     </x:row>
     <x:row r="455">
       <x:c r="A455" s="4" t="s">
+        <x:v>4237</x:v>
+      </x:c>
+      <x:c r="B455" s="4" t="s">
         <x:v>4238</x:v>
-      </x:c>
-      <x:c r="B455" s="4" t="s">
-        <x:v>4239</x:v>
       </x:c>
       <x:c r="O455" s="4" t="s">
         <x:v>2789</x:v>
@@ -35469,13 +35962,13 @@
     </x:row>
     <x:row r="456">
       <x:c r="A456" s="4" t="s">
+        <x:v>4239</x:v>
+      </x:c>
+      <x:c r="B456" s="4" t="s">
         <x:v>4240</x:v>
       </x:c>
-      <x:c r="B456" s="4" t="s">
+      <x:c r="O456" s="4" t="s">
         <x:v>4241</x:v>
-      </x:c>
-      <x:c r="O456" s="4" t="s">
-        <x:v>4242</x:v>
       </x:c>
     </x:row>
     <x:row r="458">
@@ -35491,223 +35984,448 @@
     </x:row>
     <x:row r="459">
       <x:c r="A459" s="4" t="s">
+        <x:v>4242</x:v>
+      </x:c>
+      <x:c r="B459" s="4" t="s">
         <x:v>4243</x:v>
       </x:c>
-      <x:c r="B459" s="4" t="s">
+      <x:c r="O459" s="4" t="s">
         <x:v>4244</x:v>
-      </x:c>
-      <x:c r="O459" s="4" t="s">
-        <x:v>4245</x:v>
       </x:c>
     </x:row>
     <x:row r="460">
       <x:c r="A460" s="4" t="s">
+        <x:v>4245</x:v>
+      </x:c>
+      <x:c r="B460" s="4" t="s">
         <x:v>4246</x:v>
       </x:c>
-      <x:c r="B460" s="4" t="s">
+      <x:c r="O460" s="4" t="s">
         <x:v>4247</x:v>
-      </x:c>
-      <x:c r="O460" s="4" t="s">
-        <x:v>4248</x:v>
       </x:c>
     </x:row>
     <x:row r="463">
       <x:c r="A463" s="4" t="s">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="B463" s="4" t="s">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="O463" s="4" t="s">
         <x:v>4249</x:v>
-      </x:c>
-      <x:c r="B463" s="4" t="s">
-        <x:v>4249</x:v>
-      </x:c>
-      <x:c r="O463" s="4" t="s">
-        <x:v>4250</x:v>
       </x:c>
     </x:row>
     <x:row r="464">
       <x:c r="A464" s="4" t="s">
+        <x:v>4250</x:v>
+      </x:c>
+      <x:c r="B464" s="4" t="s">
         <x:v>4251</x:v>
       </x:c>
-      <x:c r="B464" s="4" t="s">
+      <x:c r="O464" s="4" t="s">
         <x:v>4252</x:v>
-      </x:c>
-      <x:c r="O464" s="4" t="s">
-        <x:v>4253</x:v>
       </x:c>
     </x:row>
     <x:row r="465">
       <x:c r="A465" s="4" t="s">
+        <x:v>4253</x:v>
+      </x:c>
+      <x:c r="B465" s="4" t="s">
         <x:v>4254</x:v>
       </x:c>
-      <x:c r="B465" s="4" t="s">
+      <x:c r="O465" s="4" t="s">
         <x:v>4255</x:v>
-      </x:c>
-      <x:c r="O465" s="4" t="s">
-        <x:v>4256</x:v>
       </x:c>
     </x:row>
     <x:row r="467">
       <x:c r="A467" s="4" t="s">
+        <x:v>4256</x:v>
+      </x:c>
+      <x:c r="B467" s="4" t="s">
+        <x:v>4256</x:v>
+      </x:c>
+      <x:c r="O467" s="4" t="s">
         <x:v>4257</x:v>
-      </x:c>
-      <x:c r="B467" s="4" t="s">
-        <x:v>4257</x:v>
-      </x:c>
-      <x:c r="O467" s="4" t="s">
-        <x:v>4258</x:v>
       </x:c>
     </x:row>
     <x:row r="468">
       <x:c r="A468" s="4" t="s">
+        <x:v>4258</x:v>
+      </x:c>
+      <x:c r="B468" s="4" t="s">
         <x:v>4259</x:v>
       </x:c>
-      <x:c r="B468" s="4" t="s">
+      <x:c r="O468" s="4" t="s">
         <x:v>4260</x:v>
-      </x:c>
-      <x:c r="O468" s="4" t="s">
-        <x:v>4261</x:v>
       </x:c>
     </x:row>
     <x:row r="469">
       <x:c r="A469" s="4" t="s">
-        <x:v>4262</x:v>
+        <x:v>4261</x:v>
       </x:c>
       <x:c r="B469" s="4" t="s">
+        <x:v>4259</x:v>
+      </x:c>
+      <x:c r="O469" s="4" t="s">
         <x:v>4260</x:v>
-      </x:c>
-      <x:c r="O469" s="4" t="s">
-        <x:v>4261</x:v>
       </x:c>
     </x:row>
     <x:row r="471">
       <x:c r="A471" s="4" t="s">
+        <x:v>4262</x:v>
+      </x:c>
+      <x:c r="B471" s="4" t="s">
+        <x:v>4262</x:v>
+      </x:c>
+      <x:c r="O471" s="4" t="s">
         <x:v>4263</x:v>
-      </x:c>
-      <x:c r="B471" s="4" t="s">
-        <x:v>4263</x:v>
-      </x:c>
-      <x:c r="O471" s="4" t="s">
-        <x:v>4264</x:v>
       </x:c>
     </x:row>
     <x:row r="472">
       <x:c r="A472" s="4" t="s">
+        <x:v>4264</x:v>
+      </x:c>
+      <x:c r="B472" s="4" t="s">
         <x:v>4265</x:v>
       </x:c>
-      <x:c r="B472" s="4" t="s">
+      <x:c r="O472" s="4" t="s">
         <x:v>4266</x:v>
-      </x:c>
-      <x:c r="O472" s="4" t="s">
-        <x:v>4267</x:v>
       </x:c>
     </x:row>
     <x:row r="473">
       <x:c r="A473" s="4" t="s">
+        <x:v>4267</x:v>
+      </x:c>
+      <x:c r="B473" s="4" t="s">
         <x:v>4268</x:v>
       </x:c>
-      <x:c r="B473" s="4" t="s">
-        <x:v>4269</x:v>
-      </x:c>
       <x:c r="O473" s="4" t="s">
-        <x:v>4267</x:v>
+        <x:v>4266</x:v>
       </x:c>
     </x:row>
     <x:row r="475">
       <x:c r="A475" s="4" t="s">
-        <x:v>4011</x:v>
+        <x:v>4010</x:v>
       </x:c>
       <x:c r="B475" s="4" t="s">
-        <x:v>4011</x:v>
+        <x:v>4010</x:v>
       </x:c>
       <x:c r="O475" s="4" t="s">
-        <x:v>4270</x:v>
+        <x:v>4269</x:v>
       </x:c>
     </x:row>
     <x:row r="476">
       <x:c r="A476" s="4" t="s">
+        <x:v>4270</x:v>
+      </x:c>
+      <x:c r="B476" s="4" t="s">
         <x:v>4271</x:v>
       </x:c>
-      <x:c r="B476" s="4" t="s">
+      <x:c r="O476" s="4" t="s">
         <x:v>4272</x:v>
-      </x:c>
-      <x:c r="O476" s="4" t="s">
-        <x:v>4273</x:v>
       </x:c>
     </x:row>
     <x:row r="477">
       <x:c r="A477" s="4" t="s">
+        <x:v>4273</x:v>
+      </x:c>
+      <x:c r="B477" s="4" t="s">
+        <x:v>4271</x:v>
+      </x:c>
+      <x:c r="O477" s="4" t="s">
         <x:v>4274</x:v>
-      </x:c>
-      <x:c r="B477" s="4" t="s">
-        <x:v>4272</x:v>
-      </x:c>
-      <x:c r="O477" s="4" t="s">
-        <x:v>4275</x:v>
       </x:c>
     </x:row>
     <x:row r="479">
       <x:c r="A479" s="4" t="s">
+        <x:v>4275</x:v>
+      </x:c>
+      <x:c r="B479" s="4" t="s">
+        <x:v>4275</x:v>
+      </x:c>
+      <x:c r="O479" s="4" t="s">
         <x:v>4276</x:v>
-      </x:c>
-      <x:c r="B479" s="4" t="s">
-        <x:v>4276</x:v>
-      </x:c>
-      <x:c r="O479" s="4" t="s">
-        <x:v>4277</x:v>
       </x:c>
     </x:row>
     <x:row r="480">
       <x:c r="A480" s="4" t="s">
+        <x:v>4277</x:v>
+      </x:c>
+      <x:c r="B480" s="4" t="s">
         <x:v>4278</x:v>
       </x:c>
-      <x:c r="B480" s="4" t="s">
+      <x:c r="O480" s="4" t="s">
         <x:v>4279</x:v>
-      </x:c>
-      <x:c r="O480" s="4" t="s">
-        <x:v>4280</x:v>
       </x:c>
     </x:row>
     <x:row r="481">
       <x:c r="A481" s="4" t="s">
+        <x:v>4280</x:v>
+      </x:c>
+      <x:c r="B481" s="4" t="s">
         <x:v>4281</x:v>
       </x:c>
-      <x:c r="B481" s="4" t="s">
+      <x:c r="O481" s="4" t="s">
         <x:v>4282</x:v>
-      </x:c>
-      <x:c r="O481" s="4" t="s">
-        <x:v>4283</x:v>
       </x:c>
     </x:row>
     <x:row r="483">
       <x:c r="A483" s="4" t="s">
+        <x:v>4283</x:v>
+      </x:c>
+      <x:c r="B483" s="4" t="s">
         <x:v>4284</x:v>
       </x:c>
-      <x:c r="B483" s="4" t="s">
+      <x:c r="O483" s="4" t="s">
         <x:v>4285</x:v>
-      </x:c>
-      <x:c r="O483" s="4" t="s">
-        <x:v>4286</x:v>
       </x:c>
     </x:row>
     <x:row r="484">
       <x:c r="A484" s="4" t="s">
+        <x:v>4286</x:v>
+      </x:c>
+      <x:c r="B484" s="4" t="s">
         <x:v>4287</x:v>
       </x:c>
-      <x:c r="B484" s="4" t="s">
+      <x:c r="O484" s="4" t="s">
         <x:v>4288</x:v>
-      </x:c>
-      <x:c r="O484" s="4" t="s">
-        <x:v>4289</x:v>
       </x:c>
     </x:row>
     <x:row r="485">
       <x:c r="A485" s="4" t="s">
+        <x:v>4289</x:v>
+      </x:c>
+      <x:c r="B485" s="4" t="s">
         <x:v>4290</x:v>
       </x:c>
-      <x:c r="B485" s="4" t="s">
+      <x:c r="O485" s="4" t="s">
         <x:v>4291</x:v>
       </x:c>
-      <x:c r="O485" s="4" t="s">
-        <x:v>4292</x:v>
-      </x:c>
+    </x:row>
+    <x:row r="486">
+      <x:c r="A486" t="str">
+        <x:v>Imitator</x:v>
+      </x:c>
+      <x:c r="B486" t="str">
+        <x:v>Imitator</x:v>
+      </x:c>
+      <x:c r="C486"/>
+      <x:c r="D486"/>
+      <x:c r="E486"/>
+      <x:c r="F486"/>
+      <x:c r="G486"/>
+      <x:c r="H486"/>
+      <x:c r="I486"/>
+      <x:c r="J486"/>
+      <x:c r="K486"/>
+      <x:c r="L486"/>
+      <x:c r="M486"/>
+      <x:c r="N486"/>
+      <x:c r="O486" t="str">
+        <x:v>效颦者</x:v>
+      </x:c>
+      <x:c r="P486"/>
+      <x:c r="Q486"/>
+    </x:row>
+    <x:row r="487">
+      <x:c r="A487" t="str">
+        <x:v>ImitatorIntroDesc</x:v>
+      </x:c>
+      <x:c r="B487" t="str">
+        <x:v>Borrow the dead's talents.</x:v>
+      </x:c>
+      <x:c r="C487"/>
+      <x:c r="D487"/>
+      <x:c r="E487"/>
+      <x:c r="F487"/>
+      <x:c r="G487"/>
+      <x:c r="H487"/>
+      <x:c r="I487"/>
+      <x:c r="J487"/>
+      <x:c r="K487"/>
+      <x:c r="L487"/>
+      <x:c r="M487"/>
+      <x:c r="N487"/>
+      <x:c r="O487" t="str">
+        <x:v>借死者之才为己所用。</x:v>
+      </x:c>
+      <x:c r="P487"/>
+      <x:c r="Q487"/>
+    </x:row>
+    <x:row r="488">
+      <x:c r="A488" t="str">
+        <x:v>ImitatorShortDesc</x:v>
+      </x:c>
+      <x:c r="B488" t="str">
+        <x:v>Select a dead crewmate during a meeting and use their role for the next round.</x:v>
+      </x:c>
+      <x:c r="C488"/>
+      <x:c r="D488"/>
+      <x:c r="E488"/>
+      <x:c r="F488"/>
+      <x:c r="G488"/>
+      <x:c r="H488"/>
+      <x:c r="I488"/>
+      <x:c r="J488"/>
+      <x:c r="K488"/>
+      <x:c r="L488"/>
+      <x:c r="M488"/>
+      <x:c r="N488"/>
+      <x:c r="O488" t="str">
+        <x:v>在会议中选择死亡船员，并在下一行动轮使用其职业。</x:v>
+      </x:c>
+      <x:c r="P488"/>
+      <x:c r="Q488"/>
+    </x:row>
+    <x:row r="489">
+      <x:c r="A489" t="str">
+        <x:v>TrapperPlus</x:v>
+      </x:c>
+      <x:c r="B489" t="str">
+        <x:v>Trapper Plus</x:v>
+      </x:c>
+      <x:c r="C489"/>
+      <x:c r="D489"/>
+      <x:c r="E489"/>
+      <x:c r="F489"/>
+      <x:c r="G489"/>
+      <x:c r="H489"/>
+      <x:c r="I489"/>
+      <x:c r="J489"/>
+      <x:c r="K489"/>
+      <x:c r="L489"/>
+      <x:c r="M489"/>
+      <x:c r="N489"/>
+      <x:c r="O489" t="str">
+        <x:v>陷阱师</x:v>
+      </x:c>
+      <x:c r="P489"/>
+      <x:c r="Q489"/>
+    </x:row>
+    <x:row r="490">
+      <x:c r="A490" t="str">
+        <x:v>TrapperPlusIntroDesc</x:v>
+      </x:c>
+      <x:c r="B490" t="str">
+        <x:v>Learn who lingers in your traps.</x:v>
+      </x:c>
+      <x:c r="C490"/>
+      <x:c r="D490"/>
+      <x:c r="E490"/>
+      <x:c r="F490"/>
+      <x:c r="G490"/>
+      <x:c r="H490"/>
+      <x:c r="I490"/>
+      <x:c r="J490"/>
+      <x:c r="K490"/>
+      <x:c r="L490"/>
+      <x:c r="M490"/>
+      <x:c r="N490"/>
+      <x:c r="O490" t="str">
+        <x:v>从逗留在陷阱中的玩家身上获取情报。</x:v>
+      </x:c>
+      <x:c r="P490"/>
+      <x:c r="Q490"/>
+    </x:row>
+    <x:row r="491">
+      <x:c r="A491" t="str">
+        <x:v>TrapperPlusShortDesc</x:v>
+      </x:c>
+      <x:c r="B491" t="str">
+        <x:v>Place hidden information traps and receive an anonymous role report.</x:v>
+      </x:c>
+      <x:c r="C491"/>
+      <x:c r="D491"/>
+      <x:c r="E491"/>
+      <x:c r="F491"/>
+      <x:c r="G491"/>
+      <x:c r="H491"/>
+      <x:c r="I491"/>
+      <x:c r="J491"/>
+      <x:c r="K491"/>
+      <x:c r="L491"/>
+      <x:c r="M491"/>
+      <x:c r="N491"/>
+      <x:c r="O491" t="str">
+        <x:v>放置信息陷阱，并获得匿名职业报告。</x:v>
+      </x:c>
+      <x:c r="P491"/>
+      <x:c r="Q491"/>
+    </x:row>
+    <x:row r="492">
+      <x:c r="A492" t="str">
+        <x:v>Aurial</x:v>
+      </x:c>
+      <x:c r="B492" t="str">
+        <x:v>Aurial</x:v>
+      </x:c>
+      <x:c r="C492"/>
+      <x:c r="D492"/>
+      <x:c r="E492"/>
+      <x:c r="F492"/>
+      <x:c r="G492"/>
+      <x:c r="H492"/>
+      <x:c r="I492"/>
+      <x:c r="J492"/>
+      <x:c r="K492"/>
+      <x:c r="L492"/>
+      <x:c r="M492"/>
+      <x:c r="N492"/>
+      <x:c r="O492" t="str">
+        <x:v>灵光师</x:v>
+      </x:c>
+      <x:c r="P492"/>
+      <x:c r="Q492"/>
+    </x:row>
+    <x:row r="493">
+      <x:c r="A493" t="str">
+        <x:v>AurialIntroDesc</x:v>
+      </x:c>
+      <x:c r="B493" t="str">
+        <x:v>Let their factions glow.</x:v>
+      </x:c>
+      <x:c r="C493"/>
+      <x:c r="D493"/>
+      <x:c r="E493"/>
+      <x:c r="F493"/>
+      <x:c r="G493"/>
+      <x:c r="H493"/>
+      <x:c r="I493"/>
+      <x:c r="J493"/>
+      <x:c r="K493"/>
+      <x:c r="L493"/>
+      <x:c r="M493"/>
+      <x:c r="N493"/>
+      <x:c r="O493" t="str">
+        <x:v>让他们的阵营显现灵光。</x:v>
+      </x:c>
+      <x:c r="P493"/>
+      <x:c r="Q493"/>
+    </x:row>
+    <x:row r="494">
+      <x:c r="A494" t="str">
+        <x:v>AurialShortDesc</x:v>
+      </x:c>
+      <x:c r="B494" t="str">
+        <x:v>Radiate nearby players repeatedly to reveal their factions.</x:v>
+      </x:c>
+      <x:c r="C494"/>
+      <x:c r="D494"/>
+      <x:c r="E494"/>
+      <x:c r="F494"/>
+      <x:c r="G494"/>
+      <x:c r="H494"/>
+      <x:c r="I494"/>
+      <x:c r="J494"/>
+      <x:c r="K494"/>
+      <x:c r="L494"/>
+      <x:c r="M494"/>
+      <x:c r="N494"/>
+      <x:c r="O494" t="str">
+        <x:v>反复辐射附近玩家以识别其阵营。</x:v>
+      </x:c>
+      <x:c r="P494"/>
+      <x:c r="Q494"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -35782,1327 +36500,1402 @@
     </x:row>
     <x:row r="2" ht="60" customHeight="1">
       <x:c r="A2" s="1" t="s">
+        <x:v>4292</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
         <x:v>4293</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
+      <x:c r="O2" s="1" t="s">
         <x:v>4294</x:v>
-      </x:c>
-      <x:c r="O2" s="1" t="s">
-        <x:v>4295</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="60" customHeight="1">
       <x:c r="A3" s="1" t="s">
+        <x:v>4295</x:v>
+      </x:c>
+      <x:c r="B3" s="1" t="s">
         <x:v>4296</x:v>
       </x:c>
-      <x:c r="B3" s="1" t="s">
+      <x:c r="O3" s="1" t="s">
         <x:v>4297</x:v>
-      </x:c>
-      <x:c r="O3" s="1" t="s">
-        <x:v>4298</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="60" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>4298</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="s">
         <x:v>4299</x:v>
       </x:c>
-      <x:c r="B4" s="1" t="s">
+      <x:c r="O4" s="15" t="s">
         <x:v>4300</x:v>
-      </x:c>
-      <x:c r="O4" s="15" t="s">
-        <x:v>4301</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="60" customHeight="1">
       <x:c r="A5" s="15" t="s">
+        <x:v>4301</x:v>
+      </x:c>
+      <x:c r="O5" s="15" t="s">
         <x:v>4302</x:v>
-      </x:c>
-      <x:c r="O5" s="15" t="s">
-        <x:v>4303</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="60" customHeight="1">
       <x:c r="A6" s="1" t="s">
+        <x:v>4303</x:v>
+      </x:c>
+      <x:c r="B6" s="1" t="s">
         <x:v>4304</x:v>
       </x:c>
-      <x:c r="B6" s="1" t="s">
+      <x:c r="O6" s="1" t="s">
         <x:v>4305</x:v>
-      </x:c>
-      <x:c r="O6" s="1" t="s">
-        <x:v>4306</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="60" customHeight="1">
       <x:c r="A7" s="1" t="s">
+        <x:v>4306</x:v>
+      </x:c>
+      <x:c r="B7" s="1" t="s">
         <x:v>4307</x:v>
       </x:c>
-      <x:c r="B7" s="1" t="s">
+      <x:c r="O7" s="1" t="s">
         <x:v>4308</x:v>
-      </x:c>
-      <x:c r="O7" s="1" t="s">
-        <x:v>4309</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="60" customHeight="1">
       <x:c r="A8" s="1" t="s">
+        <x:v>4309</x:v>
+      </x:c>
+      <x:c r="B8" s="1" t="s">
         <x:v>4310</x:v>
       </x:c>
-      <x:c r="B8" s="1" t="s">
+      <x:c r="O8" s="1" t="s">
         <x:v>4311</x:v>
-      </x:c>
-      <x:c r="O8" s="1" t="s">
-        <x:v>4312</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="60" customHeight="1">
       <x:c r="A9" s="1" t="s">
+        <x:v>4312</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="s">
         <x:v>4313</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="s">
+      <x:c r="O9" s="1" t="s">
         <x:v>4314</x:v>
-      </x:c>
-      <x:c r="O9" s="1" t="s">
-        <x:v>4315</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="60" customHeight="1">
       <x:c r="A10" s="1" t="s">
+        <x:v>4315</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="s">
         <x:v>4316</x:v>
       </x:c>
-      <x:c r="B10" s="1" t="s">
+      <x:c r="O10" s="1" t="s">
         <x:v>4317</x:v>
-      </x:c>
-      <x:c r="O10" s="1" t="s">
-        <x:v>4318</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="60" customHeight="1">
       <x:c r="A11" s="1" t="s">
+        <x:v>4318</x:v>
+      </x:c>
+      <x:c r="B11" s="1" t="s">
         <x:v>4319</x:v>
       </x:c>
-      <x:c r="B11" s="1" t="s">
+      <x:c r="O11" s="1" t="s">
         <x:v>4320</x:v>
-      </x:c>
-      <x:c r="O11" s="1" t="s">
-        <x:v>4321</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="60" customHeight="1">
       <x:c r="A12" s="1" t="s">
+        <x:v>4321</x:v>
+      </x:c>
+      <x:c r="B12" s="1" t="s">
         <x:v>4322</x:v>
       </x:c>
-      <x:c r="B12" s="1" t="s">
+      <x:c r="O12" s="1" t="s">
         <x:v>4323</x:v>
-      </x:c>
-      <x:c r="O12" s="1" t="s">
-        <x:v>4324</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="60" customHeight="1">
       <x:c r="A13" s="1" t="s">
+        <x:v>4324</x:v>
+      </x:c>
+      <x:c r="B13" s="1" t="s">
         <x:v>4325</x:v>
       </x:c>
-      <x:c r="B13" s="1" t="s">
+      <x:c r="O13" s="1" t="s">
         <x:v>4326</x:v>
-      </x:c>
-      <x:c r="O13" s="1" t="s">
-        <x:v>4327</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
       <x:c r="A14" s="1" t="s">
+        <x:v>4327</x:v>
+      </x:c>
+      <x:c r="B14" s="1" t="s">
         <x:v>4328</x:v>
       </x:c>
-      <x:c r="B14" s="1" t="s">
+      <x:c r="O14" s="1" t="s">
         <x:v>4329</x:v>
-      </x:c>
-      <x:c r="O14" s="1" t="s">
-        <x:v>4330</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="60" customHeight="1">
       <x:c r="A15" s="1" t="s">
+        <x:v>4330</x:v>
+      </x:c>
+      <x:c r="B15" s="1" t="s">
         <x:v>4331</x:v>
       </x:c>
-      <x:c r="B15" s="1" t="s">
+      <x:c r="O15" s="1" t="s">
         <x:v>4332</x:v>
-      </x:c>
-      <x:c r="O15" s="1" t="s">
-        <x:v>4333</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="60" customHeight="1">
       <x:c r="A16" s="1" t="s">
+        <x:v>4333</x:v>
+      </x:c>
+      <x:c r="B16" s="1" t="s">
         <x:v>4334</x:v>
       </x:c>
-      <x:c r="B16" s="1" t="s">
+      <x:c r="O16" s="1" t="s">
         <x:v>4335</x:v>
-      </x:c>
-      <x:c r="O16" s="1" t="s">
-        <x:v>4336</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="60" customHeight="1">
       <x:c r="A17" s="1" t="s">
+        <x:v>4336</x:v>
+      </x:c>
+      <x:c r="B17" s="1" t="s">
         <x:v>4337</x:v>
       </x:c>
-      <x:c r="B17" s="1" t="s">
+      <x:c r="O17" s="1" t="s">
         <x:v>4338</x:v>
-      </x:c>
-      <x:c r="O17" s="1" t="s">
-        <x:v>4339</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
       <x:c r="A18" s="1" t="s">
+        <x:v>4339</x:v>
+      </x:c>
+      <x:c r="B18" s="1" t="s">
         <x:v>4340</x:v>
       </x:c>
-      <x:c r="B18" s="1" t="s">
+      <x:c r="O18" s="1" t="s">
         <x:v>4341</x:v>
-      </x:c>
-      <x:c r="O18" s="1" t="s">
-        <x:v>4342</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="60" customHeight="1">
       <x:c r="A19" s="1" t="s">
+        <x:v>4342</x:v>
+      </x:c>
+      <x:c r="B19" s="1" t="s">
         <x:v>4343</x:v>
       </x:c>
-      <x:c r="B19" s="1" t="s">
+      <x:c r="O19" s="1" t="s">
         <x:v>4344</x:v>
-      </x:c>
-      <x:c r="O19" s="1" t="s">
-        <x:v>4345</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
       <x:c r="A20" s="1" t="s">
-        <x:v>4328</x:v>
+        <x:v>4327</x:v>
       </x:c>
       <x:c r="B20" s="1" t="s">
+        <x:v>4345</x:v>
+      </x:c>
+      <x:c r="O20" s="1" t="s">
         <x:v>4346</x:v>
-      </x:c>
-      <x:c r="O20" s="1" t="s">
-        <x:v>4347</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
       <x:c r="A21" s="1" t="s">
+        <x:v>4347</x:v>
+      </x:c>
+      <x:c r="B21" s="1" t="s">
         <x:v>4348</x:v>
       </x:c>
-      <x:c r="B21" s="1" t="s">
+      <x:c r="O21" s="1" t="s">
         <x:v>4349</x:v>
-      </x:c>
-      <x:c r="O21" s="1" t="s">
-        <x:v>4350</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="60" customHeight="1">
       <x:c r="A22" s="1" t="s">
+        <x:v>4350</x:v>
+      </x:c>
+      <x:c r="B22" s="1" t="s">
         <x:v>4351</x:v>
       </x:c>
-      <x:c r="B22" s="1" t="s">
+      <x:c r="O22" s="1" t="s">
         <x:v>4352</x:v>
-      </x:c>
-      <x:c r="O22" s="1" t="s">
-        <x:v>4353</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
       <x:c r="A23" s="1" t="s">
+        <x:v>4353</x:v>
+      </x:c>
+      <x:c r="B23" s="1" t="s">
         <x:v>4354</x:v>
       </x:c>
-      <x:c r="B23" s="1" t="s">
+      <x:c r="O23" s="1" t="s">
         <x:v>4355</x:v>
-      </x:c>
-      <x:c r="O23" s="1" t="s">
-        <x:v>4356</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="60" customHeight="1">
       <x:c r="A24" s="1" t="s">
+        <x:v>4356</x:v>
+      </x:c>
+      <x:c r="B24" s="1" t="s">
         <x:v>4357</x:v>
       </x:c>
-      <x:c r="B24" s="1" t="s">
+      <x:c r="O24" s="1" t="s">
         <x:v>4358</x:v>
-      </x:c>
-      <x:c r="O24" s="1" t="s">
-        <x:v>4359</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
       <x:c r="A25" s="1" t="s">
+        <x:v>4359</x:v>
+      </x:c>
+      <x:c r="B25" s="1" t="s">
         <x:v>4360</x:v>
       </x:c>
-      <x:c r="B25" s="1" t="s">
+      <x:c r="O25" s="1" t="s">
         <x:v>4361</x:v>
-      </x:c>
-      <x:c r="O25" s="1" t="s">
-        <x:v>4362</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="60" customHeight="1">
       <x:c r="A26" s="1" t="s">
+        <x:v>4362</x:v>
+      </x:c>
+      <x:c r="B26" s="1" t="s">
         <x:v>4363</x:v>
       </x:c>
-      <x:c r="B26" s="1" t="s">
+      <x:c r="O26" s="1" t="s">
         <x:v>4364</x:v>
-      </x:c>
-      <x:c r="O26" s="1" t="s">
-        <x:v>4365</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
       <x:c r="A27" s="1" t="s">
+        <x:v>4365</x:v>
+      </x:c>
+      <x:c r="B27" s="1" t="s">
         <x:v>4366</x:v>
       </x:c>
-      <x:c r="B27" s="1" t="s">
+      <x:c r="O27" s="1" t="s">
         <x:v>4367</x:v>
-      </x:c>
-      <x:c r="O27" s="1" t="s">
-        <x:v>4368</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
       <x:c r="A28" s="1" t="s">
+        <x:v>4368</x:v>
+      </x:c>
+      <x:c r="B28" s="1" t="s">
         <x:v>4369</x:v>
       </x:c>
-      <x:c r="B28" s="1" t="s">
+      <x:c r="O28" s="1" t="s">
         <x:v>4370</x:v>
-      </x:c>
-      <x:c r="O28" s="1" t="s">
-        <x:v>4371</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="60" customHeight="1">
       <x:c r="A29" s="1" t="s">
+        <x:v>4371</x:v>
+      </x:c>
+      <x:c r="B29" s="1" t="s">
         <x:v>4372</x:v>
       </x:c>
-      <x:c r="B29" s="1" t="s">
+      <x:c r="O29" s="1" t="s">
         <x:v>4373</x:v>
-      </x:c>
-      <x:c r="O29" s="1" t="s">
-        <x:v>4374</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="60" customHeight="1">
       <x:c r="A30" s="1" t="s">
+        <x:v>4374</x:v>
+      </x:c>
+      <x:c r="B30" s="1" t="s">
         <x:v>4375</x:v>
       </x:c>
-      <x:c r="B30" s="1" t="s">
+      <x:c r="O30" s="1" t="s">
         <x:v>4376</x:v>
-      </x:c>
-      <x:c r="O30" s="1" t="s">
-        <x:v>4377</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="60" customHeight="1">
       <x:c r="A31" s="1" t="s">
+        <x:v>4377</x:v>
+      </x:c>
+      <x:c r="B31" s="1" t="s">
         <x:v>4378</x:v>
       </x:c>
-      <x:c r="B31" s="1" t="s">
+      <x:c r="O31" s="1" t="s">
         <x:v>4379</x:v>
-      </x:c>
-      <x:c r="O31" s="1" t="s">
-        <x:v>4380</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="60" customHeight="1">
       <x:c r="A32" s="1" t="s">
+        <x:v>4380</x:v>
+      </x:c>
+      <x:c r="B32" s="1" t="s">
         <x:v>4381</x:v>
       </x:c>
-      <x:c r="B32" s="1" t="s">
+      <x:c r="O32" s="1" t="s">
         <x:v>4382</x:v>
-      </x:c>
-      <x:c r="O32" s="1" t="s">
-        <x:v>4383</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="60" customHeight="1">
       <x:c r="A34" s="1" t="s">
+        <x:v>4383</x:v>
+      </x:c>
+      <x:c r="B34" s="1" t="s">
         <x:v>4384</x:v>
       </x:c>
-      <x:c r="B34" s="1" t="s">
+      <x:c r="O34" s="1" t="s">
         <x:v>4385</x:v>
-      </x:c>
-      <x:c r="O34" s="1" t="s">
-        <x:v>4386</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="60" customHeight="1">
       <x:c r="A35" s="1" t="s">
+        <x:v>4386</x:v>
+      </x:c>
+      <x:c r="B35" s="1" t="s">
         <x:v>4387</x:v>
       </x:c>
-      <x:c r="B35" s="1" t="s">
+      <x:c r="O35" s="1" t="s">
         <x:v>4388</x:v>
-      </x:c>
-      <x:c r="O35" s="1" t="s">
-        <x:v>4389</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="60" customHeight="1">
       <x:c r="A36" s="1" t="s">
+        <x:v>4389</x:v>
+      </x:c>
+      <x:c r="B36" s="1" t="s">
         <x:v>4390</x:v>
       </x:c>
-      <x:c r="B36" s="1" t="s">
+      <x:c r="O36" s="1" t="s">
         <x:v>4391</x:v>
-      </x:c>
-      <x:c r="O36" s="1" t="s">
-        <x:v>4392</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="60" customHeight="1">
       <x:c r="A37" s="1" t="s">
+        <x:v>4392</x:v>
+      </x:c>
+      <x:c r="B37" s="3" t="s">
         <x:v>4393</x:v>
       </x:c>
-      <x:c r="B37" s="3" t="s">
+      <x:c r="O37" s="1" t="s">
         <x:v>4394</x:v>
-      </x:c>
-      <x:c r="O37" s="1" t="s">
-        <x:v>4395</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="60" customHeight="1">
       <x:c r="A38" s="1" t="s">
+        <x:v>4395</x:v>
+      </x:c>
+      <x:c r="B38" s="1" t="s">
         <x:v>4396</x:v>
       </x:c>
-      <x:c r="B38" s="1" t="s">
+      <x:c r="O38" s="1" t="s">
         <x:v>4397</x:v>
-      </x:c>
-      <x:c r="O38" s="1" t="s">
-        <x:v>4398</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="60" customHeight="1">
       <x:c r="A39" s="1" t="s">
+        <x:v>4398</x:v>
+      </x:c>
+      <x:c r="B39" s="1" t="s">
         <x:v>4399</x:v>
       </x:c>
-      <x:c r="B39" s="1" t="s">
+      <x:c r="O39" s="1" t="s">
         <x:v>4400</x:v>
-      </x:c>
-      <x:c r="O39" s="1" t="s">
-        <x:v>4401</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="60" customHeight="1">
       <x:c r="A40" s="1" t="s">
+        <x:v>4401</x:v>
+      </x:c>
+      <x:c r="B40" s="1" t="s">
         <x:v>4402</x:v>
       </x:c>
-      <x:c r="B40" s="1" t="s">
+      <x:c r="O40" s="1" t="s">
         <x:v>4403</x:v>
-      </x:c>
-      <x:c r="O40" s="1" t="s">
-        <x:v>4404</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="60" customHeight="1">
       <x:c r="A41" s="1" t="s">
+        <x:v>4404</x:v>
+      </x:c>
+      <x:c r="B41" s="1" t="s">
         <x:v>4405</x:v>
       </x:c>
-      <x:c r="B41" s="1" t="s">
+      <x:c r="O41" s="1" t="s">
         <x:v>4406</x:v>
-      </x:c>
-      <x:c r="O41" s="1" t="s">
-        <x:v>4407</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="60" customHeight="1">
       <x:c r="A42" s="1" t="s">
+        <x:v>4407</x:v>
+      </x:c>
+      <x:c r="B42" s="1" t="s">
         <x:v>4408</x:v>
       </x:c>
-      <x:c r="B42" s="1" t="s">
+      <x:c r="O42" s="1" t="s">
         <x:v>4409</x:v>
-      </x:c>
-      <x:c r="O42" s="1" t="s">
-        <x:v>4410</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="60" customHeight="1">
       <x:c r="A43" s="1" t="s">
+        <x:v>4410</x:v>
+      </x:c>
+      <x:c r="B43" s="1" t="s">
         <x:v>4411</x:v>
       </x:c>
-      <x:c r="B43" s="1" t="s">
+      <x:c r="O43" s="1" t="s">
         <x:v>4412</x:v>
-      </x:c>
-      <x:c r="O43" s="1" t="s">
-        <x:v>4413</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="60" customHeight="1">
       <x:c r="A44" s="1" t="s">
+        <x:v>4413</x:v>
+      </x:c>
+      <x:c r="B44" s="1" t="s">
         <x:v>4414</x:v>
       </x:c>
-      <x:c r="B44" s="1" t="s">
+      <x:c r="O44" s="1" t="s">
         <x:v>4415</x:v>
-      </x:c>
-      <x:c r="O44" s="1" t="s">
-        <x:v>4416</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="60" customHeight="1">
       <x:c r="A45" s="1" t="s">
+        <x:v>4416</x:v>
+      </x:c>
+      <x:c r="B45" s="1" t="s">
         <x:v>4417</x:v>
       </x:c>
-      <x:c r="B45" s="1" t="s">
+      <x:c r="O45" s="1" t="s">
         <x:v>4418</x:v>
-      </x:c>
-      <x:c r="O45" s="1" t="s">
-        <x:v>4419</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="85.5">
       <x:c r="A46" s="1" t="s">
+        <x:v>4419</x:v>
+      </x:c>
+      <x:c r="B46" s="1" t="s">
         <x:v>4420</x:v>
       </x:c>
-      <x:c r="B46" s="1" t="s">
+      <x:c r="O46" s="1" t="s">
         <x:v>4421</x:v>
-      </x:c>
-      <x:c r="O46" s="1" t="s">
-        <x:v>4422</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="60" customHeight="1">
       <x:c r="A47" s="1" t="s">
+        <x:v>4422</x:v>
+      </x:c>
+      <x:c r="B47" s="1" t="s">
         <x:v>4423</x:v>
       </x:c>
-      <x:c r="B47" s="1" t="s">
+      <x:c r="O47" s="1" t="s">
         <x:v>4424</x:v>
-      </x:c>
-      <x:c r="O47" s="1" t="s">
-        <x:v>4425</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="60" customHeight="1">
       <x:c r="A48" s="1" t="s">
+        <x:v>4425</x:v>
+      </x:c>
+      <x:c r="B48" s="1" t="s">
         <x:v>4426</x:v>
       </x:c>
-      <x:c r="B48" s="1" t="s">
+      <x:c r="O48" s="1" t="s">
         <x:v>4427</x:v>
-      </x:c>
-      <x:c r="O48" s="1" t="s">
-        <x:v>4428</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="60" customHeight="1">
       <x:c r="A49" s="1" t="s">
+        <x:v>4428</x:v>
+      </x:c>
+      <x:c r="B49" s="1" t="s">
         <x:v>4429</x:v>
       </x:c>
-      <x:c r="B49" s="1" t="s">
+      <x:c r="O49" s="1" t="s">
         <x:v>4430</x:v>
-      </x:c>
-      <x:c r="O49" s="1" t="s">
-        <x:v>4431</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="60" customHeight="1">
       <x:c r="A50" s="1" t="s">
+        <x:v>4431</x:v>
+      </x:c>
+      <x:c r="B50" s="1" t="s">
         <x:v>4432</x:v>
       </x:c>
-      <x:c r="B50" s="1" t="s">
+      <x:c r="O50" s="1" t="s">
         <x:v>4433</x:v>
-      </x:c>
-      <x:c r="O50" s="1" t="s">
-        <x:v>4434</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="60" customHeight="1">
       <x:c r="A51" s="1" t="s">
+        <x:v>4434</x:v>
+      </x:c>
+      <x:c r="B51" s="1" t="s">
         <x:v>4435</x:v>
       </x:c>
-      <x:c r="B51" s="1" t="s">
+      <x:c r="O51" s="1" t="s">
         <x:v>4436</x:v>
-      </x:c>
-      <x:c r="O51" s="1" t="s">
-        <x:v>4437</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="60" customHeight="1">
       <x:c r="A52" s="1" t="s">
+        <x:v>4437</x:v>
+      </x:c>
+      <x:c r="B52" s="1" t="s">
         <x:v>4438</x:v>
       </x:c>
-      <x:c r="B52" s="1" t="s">
+      <x:c r="O52" s="15" t="s">
         <x:v>4439</x:v>
-      </x:c>
-      <x:c r="O52" s="15" t="s">
-        <x:v>4440</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="60" customHeight="1">
       <x:c r="A53" s="1" t="s">
+        <x:v>4440</x:v>
+      </x:c>
+      <x:c r="B53" s="1" t="s">
         <x:v>4441</x:v>
       </x:c>
-      <x:c r="B53" s="1" t="s">
+      <x:c r="O53" s="15" t="s">
         <x:v>4442</x:v>
-      </x:c>
-      <x:c r="O53" s="15" t="s">
-        <x:v>4443</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="60" customHeight="1">
       <x:c r="A54" s="1" t="s">
+        <x:v>4443</x:v>
+      </x:c>
+      <x:c r="B54" s="1" t="s">
         <x:v>4444</x:v>
       </x:c>
-      <x:c r="B54" s="1" t="s">
+      <x:c r="O54" s="15" t="s">
         <x:v>4445</x:v>
-      </x:c>
-      <x:c r="O54" s="15" t="s">
-        <x:v>4446</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="60" customHeight="1">
       <x:c r="A55" s="1" t="s">
+        <x:v>4446</x:v>
+      </x:c>
+      <x:c r="B55" s="1" t="s">
         <x:v>4447</x:v>
       </x:c>
-      <x:c r="B55" s="1" t="s">
+      <x:c r="O55" s="15" t="s">
         <x:v>4448</x:v>
-      </x:c>
-      <x:c r="O55" s="15" t="s">
-        <x:v>4449</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="132.75" customHeight="1">
       <x:c r="A56" s="1" t="s">
+        <x:v>4449</x:v>
+      </x:c>
+      <x:c r="B56" s="1" t="s">
         <x:v>4450</x:v>
       </x:c>
-      <x:c r="B56" s="1" t="s">
+      <x:c r="O56" s="15" t="s">
         <x:v>4451</x:v>
-      </x:c>
-      <x:c r="O56" s="15" t="s">
-        <x:v>4452</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="60" customHeight="1">
       <x:c r="A57" s="1" t="s">
+        <x:v>4452</x:v>
+      </x:c>
+      <x:c r="B57" s="1" t="s">
         <x:v>4453</x:v>
       </x:c>
-      <x:c r="B57" s="1" t="s">
+      <x:c r="O57" s="15" t="s">
         <x:v>4454</x:v>
-      </x:c>
-      <x:c r="O57" s="15" t="s">
-        <x:v>4455</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="60" customHeight="1">
       <x:c r="A59" s="1" t="s">
+        <x:v>4455</x:v>
+      </x:c>
+      <x:c r="B59" s="1" t="s">
         <x:v>4456</x:v>
       </x:c>
-      <x:c r="B59" s="1" t="s">
+      <x:c r="O59" s="1" t="s">
         <x:v>4457</x:v>
-      </x:c>
-      <x:c r="O59" s="1" t="s">
-        <x:v>4458</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="60" customHeight="1">
       <x:c r="A60" s="1" t="s">
+        <x:v>4458</x:v>
+      </x:c>
+      <x:c r="B60" s="1" t="s">
         <x:v>4459</x:v>
       </x:c>
-      <x:c r="B60" s="1" t="s">
+      <x:c r="O60" s="1" t="s">
         <x:v>4460</x:v>
-      </x:c>
-      <x:c r="O60" s="1" t="s">
-        <x:v>4461</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="60" customHeight="1">
       <x:c r="A61" s="1" t="s">
+        <x:v>4461</x:v>
+      </x:c>
+      <x:c r="B61" s="1" t="s">
         <x:v>4462</x:v>
       </x:c>
-      <x:c r="B61" s="1" t="s">
+      <x:c r="O61" s="1" t="s">
         <x:v>4463</x:v>
-      </x:c>
-      <x:c r="O61" s="1" t="s">
-        <x:v>4464</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="60" customHeight="1">
       <x:c r="A62" s="1" t="s">
+        <x:v>4464</x:v>
+      </x:c>
+      <x:c r="B62" s="1" t="s">
         <x:v>4465</x:v>
       </x:c>
-      <x:c r="B62" s="1" t="s">
+      <x:c r="O62" s="1" t="s">
         <x:v>4466</x:v>
-      </x:c>
-      <x:c r="O62" s="1" t="s">
-        <x:v>4467</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="60" customHeight="1">
       <x:c r="A63" s="1" t="s">
+        <x:v>4467</x:v>
+      </x:c>
+      <x:c r="B63" s="1" t="s">
         <x:v>4468</x:v>
       </x:c>
-      <x:c r="B63" s="1" t="s">
+      <x:c r="O63" s="1" t="s">
         <x:v>4469</x:v>
-      </x:c>
-      <x:c r="O63" s="1" t="s">
-        <x:v>4470</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="60" customHeight="1">
       <x:c r="A64" s="1" t="s">
+        <x:v>4470</x:v>
+      </x:c>
+      <x:c r="B64" s="1" t="s">
         <x:v>4471</x:v>
       </x:c>
-      <x:c r="B64" s="1" t="s">
+      <x:c r="O64" s="1" t="s">
         <x:v>4472</x:v>
-      </x:c>
-      <x:c r="O64" s="1" t="s">
-        <x:v>4473</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="60" customHeight="1">
       <x:c r="A65" s="1" t="s">
+        <x:v>4473</x:v>
+      </x:c>
+      <x:c r="B65" s="1" t="s">
         <x:v>4474</x:v>
       </x:c>
-      <x:c r="B65" s="1" t="s">
+      <x:c r="O65" s="1" t="s">
         <x:v>4475</x:v>
-      </x:c>
-      <x:c r="O65" s="1" t="s">
-        <x:v>4476</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="60" customHeight="1">
       <x:c r="A66" s="1" t="s">
+        <x:v>4476</x:v>
+      </x:c>
+      <x:c r="B66" s="1" t="s">
         <x:v>4477</x:v>
       </x:c>
-      <x:c r="B66" s="1" t="s">
+      <x:c r="O66" s="1" t="s">
         <x:v>4478</x:v>
-      </x:c>
-      <x:c r="O66" s="1" t="s">
-        <x:v>4479</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="60" customHeight="1">
       <x:c r="A67" s="1" t="s">
+        <x:v>4479</x:v>
+      </x:c>
+      <x:c r="B67" s="1" t="s">
         <x:v>4480</x:v>
       </x:c>
-      <x:c r="B67" s="1" t="s">
+      <x:c r="O67" s="1" t="s">
         <x:v>4481</x:v>
-      </x:c>
-      <x:c r="O67" s="1" t="s">
-        <x:v>4482</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="60" customHeight="1">
       <x:c r="A68" s="1" t="s">
+        <x:v>4482</x:v>
+      </x:c>
+      <x:c r="B68" s="1" t="s">
         <x:v>4483</x:v>
       </x:c>
-      <x:c r="B68" s="1" t="s">
+      <x:c r="O68" s="1" t="s">
         <x:v>4484</x:v>
-      </x:c>
-      <x:c r="O68" s="1" t="s">
-        <x:v>4485</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="60" customHeight="1">
       <x:c r="A69" s="1" t="s">
+        <x:v>4485</x:v>
+      </x:c>
+      <x:c r="B69" s="1" t="s">
         <x:v>4486</x:v>
       </x:c>
-      <x:c r="B69" s="1" t="s">
+      <x:c r="O69" s="1" t="s">
         <x:v>4487</x:v>
-      </x:c>
-      <x:c r="O69" s="1" t="s">
-        <x:v>4488</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="60" customHeight="1">
       <x:c r="A70" s="1" t="s">
+        <x:v>4488</x:v>
+      </x:c>
+      <x:c r="B70" s="1" t="s">
         <x:v>4489</x:v>
       </x:c>
-      <x:c r="B70" s="1" t="s">
+      <x:c r="O70" s="1" t="s">
         <x:v>4490</x:v>
-      </x:c>
-      <x:c r="O70" s="1" t="s">
-        <x:v>4491</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="60" customHeight="1">
       <x:c r="A71" s="1" t="s">
+        <x:v>4491</x:v>
+      </x:c>
+      <x:c r="B71" s="1" t="s">
         <x:v>4492</x:v>
       </x:c>
-      <x:c r="B71" s="1" t="s">
+      <x:c r="O71" s="1" t="s">
         <x:v>4493</x:v>
-      </x:c>
-      <x:c r="O71" s="1" t="s">
-        <x:v>4494</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="60" customHeight="1">
       <x:c r="A72" s="1" t="s">
+        <x:v>4494</x:v>
+      </x:c>
+      <x:c r="B72" s="1" t="s">
         <x:v>4495</x:v>
       </x:c>
-      <x:c r="B72" s="1" t="s">
+      <x:c r="O72" s="1" t="s">
         <x:v>4496</x:v>
-      </x:c>
-      <x:c r="O72" s="1" t="s">
-        <x:v>4497</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="60" customHeight="1">
       <x:c r="A73" s="1" t="s">
+        <x:v>4497</x:v>
+      </x:c>
+      <x:c r="B73" s="1" t="s">
         <x:v>4498</x:v>
       </x:c>
-      <x:c r="B73" s="1" t="s">
+      <x:c r="O73" s="1" t="s">
         <x:v>4499</x:v>
-      </x:c>
-      <x:c r="O73" s="1" t="s">
-        <x:v>4500</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="60" customHeight="1">
       <x:c r="A74" s="1" t="s">
+        <x:v>4500</x:v>
+      </x:c>
+      <x:c r="B74" s="1" t="s">
         <x:v>4501</x:v>
       </x:c>
-      <x:c r="B74" s="1" t="s">
+      <x:c r="O74" s="1" t="s">
         <x:v>4502</x:v>
-      </x:c>
-      <x:c r="O74" s="1" t="s">
-        <x:v>4503</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="60" customHeight="1">
       <x:c r="A75" s="1" t="s">
+        <x:v>4503</x:v>
+      </x:c>
+      <x:c r="B75" s="1" t="s">
         <x:v>4504</x:v>
       </x:c>
-      <x:c r="B75" s="1" t="s">
+      <x:c r="O75" s="1" t="s">
         <x:v>4505</x:v>
-      </x:c>
-      <x:c r="O75" s="1" t="s">
-        <x:v>4506</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="60" customHeight="1">
       <x:c r="A76" s="1" t="s">
+        <x:v>4506</x:v>
+      </x:c>
+      <x:c r="B76" s="1" t="s">
         <x:v>4507</x:v>
       </x:c>
-      <x:c r="B76" s="1" t="s">
+      <x:c r="O76" s="1" t="s">
         <x:v>4508</x:v>
-      </x:c>
-      <x:c r="O76" s="1" t="s">
-        <x:v>4509</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="60" customHeight="1">
       <x:c r="A77" s="1" t="s">
+        <x:v>4509</x:v>
+      </x:c>
+      <x:c r="B77" s="1" t="s">
         <x:v>4510</x:v>
       </x:c>
-      <x:c r="B77" s="1" t="s">
+      <x:c r="O77" s="1" t="s">
         <x:v>4511</x:v>
-      </x:c>
-      <x:c r="O77" s="1" t="s">
-        <x:v>4512</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="60" customHeight="1">
       <x:c r="A78" s="1" t="s">
+        <x:v>4512</x:v>
+      </x:c>
+      <x:c r="B78" s="1" t="s">
         <x:v>4513</x:v>
       </x:c>
-      <x:c r="B78" s="1" t="s">
+      <x:c r="O78" s="1" t="s">
         <x:v>4514</x:v>
-      </x:c>
-      <x:c r="O78" s="1" t="s">
-        <x:v>4515</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="60" customHeight="1">
       <x:c r="A79" s="1" t="s">
+        <x:v>4515</x:v>
+      </x:c>
+      <x:c r="B79" s="1" t="s">
         <x:v>4516</x:v>
       </x:c>
-      <x:c r="B79" s="1" t="s">
+      <x:c r="O79" s="1" t="s">
         <x:v>4517</x:v>
-      </x:c>
-      <x:c r="O79" s="1" t="s">
-        <x:v>4518</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="60" customHeight="1">
       <x:c r="A80" s="1" t="s">
+        <x:v>4518</x:v>
+      </x:c>
+      <x:c r="B80" s="1" t="s">
         <x:v>4519</x:v>
       </x:c>
-      <x:c r="B80" s="1" t="s">
+      <x:c r="O80" s="1" t="s">
         <x:v>4520</x:v>
-      </x:c>
-      <x:c r="O80" s="1" t="s">
-        <x:v>4521</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="60" customHeight="1">
       <x:c r="A81" s="1" t="s">
+        <x:v>4521</x:v>
+      </x:c>
+      <x:c r="B81" s="1" t="s">
         <x:v>4522</x:v>
       </x:c>
-      <x:c r="B81" s="1" t="s">
+      <x:c r="O81" s="1" t="s">
         <x:v>4523</x:v>
-      </x:c>
-      <x:c r="O81" s="1" t="s">
-        <x:v>4524</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="60" customHeight="1">
       <x:c r="A82" s="1" t="s">
+        <x:v>4524</x:v>
+      </x:c>
+      <x:c r="B82" s="1" t="s">
         <x:v>4525</x:v>
       </x:c>
-      <x:c r="B82" s="1" t="s">
+      <x:c r="O82" s="1" t="s">
         <x:v>4526</x:v>
-      </x:c>
-      <x:c r="O82" s="1" t="s">
-        <x:v>4527</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="60" customHeight="1">
       <x:c r="A83" s="1" t="s">
+        <x:v>4527</x:v>
+      </x:c>
+      <x:c r="B83" s="1" t="s">
         <x:v>4528</x:v>
       </x:c>
-      <x:c r="B83" s="1" t="s">
+      <x:c r="O83" s="1" t="s">
         <x:v>4529</x:v>
-      </x:c>
-      <x:c r="O83" s="1" t="s">
-        <x:v>4530</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="60" customHeight="1">
       <x:c r="A84" s="1" t="s">
+        <x:v>4530</x:v>
+      </x:c>
+      <x:c r="B84" s="1" t="s">
         <x:v>4531</x:v>
       </x:c>
-      <x:c r="B84" s="1" t="s">
+      <x:c r="O84" s="1" t="s">
         <x:v>4532</x:v>
-      </x:c>
-      <x:c r="O84" s="1" t="s">
-        <x:v>4533</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="60" customHeight="1">
       <x:c r="A85" s="1" t="s">
+        <x:v>4533</x:v>
+      </x:c>
+      <x:c r="O85" s="1" t="s">
         <x:v>4534</x:v>
-      </x:c>
-      <x:c r="O85" s="1" t="s">
-        <x:v>4535</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="60" customHeight="1">
       <x:c r="A86" s="1" t="s">
+        <x:v>4535</x:v>
+      </x:c>
+      <x:c r="B86" s="1" t="s">
         <x:v>4536</x:v>
       </x:c>
-      <x:c r="B86" s="1" t="s">
+      <x:c r="O86" s="1" t="s">
         <x:v>4537</x:v>
-      </x:c>
-      <x:c r="O86" s="1" t="s">
-        <x:v>4538</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="60" customHeight="1">
       <x:c r="A87" s="1" t="s">
+        <x:v>4538</x:v>
+      </x:c>
+      <x:c r="B87" s="1" t="s">
         <x:v>4539</x:v>
       </x:c>
-      <x:c r="B87" s="1" t="s">
+      <x:c r="O87" s="1" t="s">
         <x:v>4540</x:v>
-      </x:c>
-      <x:c r="O87" s="1" t="s">
-        <x:v>4541</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="60" customHeight="1">
       <x:c r="A88" s="15" t="s">
+        <x:v>4541</x:v>
+      </x:c>
+      <x:c r="B88" s="1" t="s">
         <x:v>4542</x:v>
       </x:c>
-      <x:c r="B88" s="1" t="s">
+      <x:c r="O88" s="1" t="s">
         <x:v>4543</x:v>
-      </x:c>
-      <x:c r="O88" s="1" t="s">
-        <x:v>4544</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="60" customHeight="1">
       <x:c r="A89" s="15" t="s">
+        <x:v>4544</x:v>
+      </x:c>
+      <x:c r="O89" s="15" t="s">
         <x:v>4545</x:v>
-      </x:c>
-      <x:c r="O89" s="15" t="s">
-        <x:v>4546</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="60" customHeight="1">
       <x:c r="A90" s="1" t="s">
+        <x:v>4546</x:v>
+      </x:c>
+      <x:c r="B90" s="1" t="s">
         <x:v>4547</x:v>
       </x:c>
-      <x:c r="B90" s="1" t="s">
+      <x:c r="O90" s="15" t="s">
         <x:v>4548</x:v>
-      </x:c>
-      <x:c r="O90" s="15" t="s">
-        <x:v>4549</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="60" customHeight="1">
       <x:c r="A91" s="1" t="s">
+        <x:v>4549</x:v>
+      </x:c>
+      <x:c r="O91" s="15" t="s">
         <x:v>4550</x:v>
-      </x:c>
-      <x:c r="O91" s="15" t="s">
-        <x:v>4551</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="60" customHeight="1">
       <x:c r="A92" s="1" t="s">
+        <x:v>4551</x:v>
+      </x:c>
+      <x:c r="B92" s="1" t="s">
         <x:v>4552</x:v>
       </x:c>
-      <x:c r="B92" s="1" t="s">
+      <x:c r="O92" s="1" t="s">
         <x:v>4553</x:v>
-      </x:c>
-      <x:c r="O92" s="1" t="s">
-        <x:v>4554</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="60" customHeight="1">
       <x:c r="A93" s="1" t="s">
+        <x:v>4554</x:v>
+      </x:c>
+      <x:c r="B93" s="1" t="s">
         <x:v>4555</x:v>
       </x:c>
-      <x:c r="B93" s="1" t="s">
+      <x:c r="O93" s="1" t="s">
         <x:v>4556</x:v>
-      </x:c>
-      <x:c r="O93" s="1" t="s">
-        <x:v>4557</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="60" customHeight="1">
       <x:c r="A94" s="1" t="s">
+        <x:v>4557</x:v>
+      </x:c>
+      <x:c r="B94" s="1" t="s">
         <x:v>4558</x:v>
       </x:c>
-      <x:c r="B94" s="1" t="s">
+      <x:c r="O94" s="1" t="s">
         <x:v>4559</x:v>
-      </x:c>
-      <x:c r="O94" s="1" t="s">
-        <x:v>4560</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="60" customHeight="1">
       <x:c r="A95" s="1" t="s">
+        <x:v>4560</x:v>
+      </x:c>
+      <x:c r="O95" s="1" t="s">
         <x:v>4561</x:v>
-      </x:c>
-      <x:c r="O95" s="1" t="s">
-        <x:v>4562</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="60" customHeight="1">
       <x:c r="A96" s="1" t="s">
+        <x:v>4562</x:v>
+      </x:c>
+      <x:c r="B96" s="1" t="s">
         <x:v>4563</x:v>
       </x:c>
-      <x:c r="B96" s="1" t="s">
+      <x:c r="O96" s="1" t="s">
         <x:v>4564</x:v>
-      </x:c>
-      <x:c r="O96" s="1" t="s">
-        <x:v>4565</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="60" customHeight="1">
       <x:c r="A97" s="1" t="s">
+        <x:v>4565</x:v>
+      </x:c>
+      <x:c r="B97" s="1" t="s">
         <x:v>4566</x:v>
       </x:c>
-      <x:c r="B97" s="1" t="s">
+      <x:c r="O97" s="1" t="s">
         <x:v>4567</x:v>
-      </x:c>
-      <x:c r="O97" s="1" t="s">
-        <x:v>4568</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="60" customHeight="1">
       <x:c r="A98" s="1" t="s">
+        <x:v>4568</x:v>
+      </x:c>
+      <x:c r="B98" s="1" t="s">
         <x:v>4569</x:v>
       </x:c>
-      <x:c r="B98" s="1" t="s">
+      <x:c r="O98" s="1" t="s">
         <x:v>4570</x:v>
-      </x:c>
-      <x:c r="O98" s="1" t="s">
-        <x:v>4571</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="60" customHeight="1">
       <x:c r="A99" s="1" t="s">
+        <x:v>4571</x:v>
+      </x:c>
+      <x:c r="B99" s="1" t="s">
         <x:v>4572</x:v>
       </x:c>
-      <x:c r="B99" s="1" t="s">
+      <x:c r="O99" s="1" t="s">
         <x:v>4573</x:v>
-      </x:c>
-      <x:c r="O99" s="1" t="s">
-        <x:v>4574</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="60" customHeight="1">
       <x:c r="A100" s="1" t="s">
+        <x:v>4574</x:v>
+      </x:c>
+      <x:c r="B100" s="1" t="s">
         <x:v>4575</x:v>
       </x:c>
-      <x:c r="B100" s="1" t="s">
+      <x:c r="O100" s="1" t="s">
         <x:v>4576</x:v>
-      </x:c>
-      <x:c r="O100" s="1" t="s">
-        <x:v>4577</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="60" customHeight="1">
       <x:c r="A101" s="1" t="s">
+        <x:v>4577</x:v>
+      </x:c>
+      <x:c r="B101" s="1" t="s">
         <x:v>4578</x:v>
       </x:c>
-      <x:c r="B101" s="1" t="s">
+      <x:c r="O101" s="1" t="s">
         <x:v>4579</x:v>
-      </x:c>
-      <x:c r="O101" s="1" t="s">
-        <x:v>4580</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="60" customHeight="1">
       <x:c r="A102" s="1" t="s">
+        <x:v>4580</x:v>
+      </x:c>
+      <x:c r="B102" s="1" t="s">
         <x:v>4581</x:v>
       </x:c>
-      <x:c r="B102" s="1" t="s">
+      <x:c r="O102" s="1" t="s">
         <x:v>4582</x:v>
-      </x:c>
-      <x:c r="O102" s="1" t="s">
-        <x:v>4583</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="60" customHeight="1">
       <x:c r="A103" s="1" t="s">
+        <x:v>4583</x:v>
+      </x:c>
+      <x:c r="B103" s="1" t="s">
         <x:v>4584</x:v>
       </x:c>
-      <x:c r="B103" s="1" t="s">
+      <x:c r="O103" s="1" t="s">
         <x:v>4585</x:v>
-      </x:c>
-      <x:c r="O103" s="1" t="s">
-        <x:v>4586</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="60" customHeight="1">
       <x:c r="A104" s="1" t="s">
+        <x:v>4586</x:v>
+      </x:c>
+      <x:c r="B104" s="1" t="s">
         <x:v>4587</x:v>
       </x:c>
-      <x:c r="B104" s="1" t="s">
+      <x:c r="O104" s="1" t="s">
         <x:v>4588</x:v>
-      </x:c>
-      <x:c r="O104" s="1" t="s">
-        <x:v>4589</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="60" customHeight="1">
       <x:c r="A105" s="1" t="s">
+        <x:v>4589</x:v>
+      </x:c>
+      <x:c r="B105" s="1" t="s">
         <x:v>4590</x:v>
       </x:c>
-      <x:c r="B105" s="1" t="s">
+      <x:c r="O105" s="1" t="s">
         <x:v>4591</x:v>
-      </x:c>
-      <x:c r="O105" s="1" t="s">
-        <x:v>4592</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="60" customHeight="1">
       <x:c r="A106" s="1" t="s">
+        <x:v>4592</x:v>
+      </x:c>
+      <x:c r="B106" s="1" t="s">
         <x:v>4593</x:v>
       </x:c>
-      <x:c r="B106" s="1" t="s">
+      <x:c r="O106" s="1" t="s">
         <x:v>4594</x:v>
-      </x:c>
-      <x:c r="O106" s="1" t="s">
-        <x:v>4595</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="60" customHeight="1">
       <x:c r="A107" s="1" t="s">
+        <x:v>4595</x:v>
+      </x:c>
+      <x:c r="B107" s="1" t="s">
         <x:v>4596</x:v>
       </x:c>
-      <x:c r="B107" s="1" t="s">
+      <x:c r="O107" s="1" t="s">
         <x:v>4597</x:v>
-      </x:c>
-      <x:c r="O107" s="1" t="s">
-        <x:v>4598</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="60" customHeight="1">
       <x:c r="A108" s="1" t="s">
+        <x:v>4598</x:v>
+      </x:c>
+      <x:c r="B108" s="1" t="s">
         <x:v>4599</x:v>
       </x:c>
-      <x:c r="B108" s="1" t="s">
+      <x:c r="O108" s="1" t="s">
         <x:v>4600</x:v>
-      </x:c>
-      <x:c r="O108" s="1" t="s">
-        <x:v>4601</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="60" customHeight="1">
       <x:c r="A109" s="1" t="s">
+        <x:v>4601</x:v>
+      </x:c>
+      <x:c r="B109" s="1" t="s">
         <x:v>4602</x:v>
       </x:c>
-      <x:c r="B109" s="1" t="s">
+      <x:c r="O109" s="1" t="s">
         <x:v>4603</x:v>
-      </x:c>
-      <x:c r="O109" s="1" t="s">
-        <x:v>4604</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="60" customHeight="1">
       <x:c r="A110" s="1" t="s">
+        <x:v>4604</x:v>
+      </x:c>
+      <x:c r="B110" s="1" t="s">
         <x:v>4605</x:v>
       </x:c>
-      <x:c r="B110" s="1" t="s">
+      <x:c r="O110" s="1" t="s">
         <x:v>4606</x:v>
-      </x:c>
-      <x:c r="O110" s="1" t="s">
-        <x:v>4607</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="60" customHeight="1">
       <x:c r="A111" s="1" t="s">
+        <x:v>4607</x:v>
+      </x:c>
+      <x:c r="B111" s="1" t="s">
         <x:v>4608</x:v>
       </x:c>
-      <x:c r="B111" s="1" t="s">
+      <x:c r="O111" s="1" t="s">
         <x:v>4609</x:v>
-      </x:c>
-      <x:c r="O111" s="1" t="s">
-        <x:v>4610</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="60" customHeight="1">
       <x:c r="A112" s="1" t="s">
+        <x:v>4610</x:v>
+      </x:c>
+      <x:c r="B112" s="1" t="s">
         <x:v>4611</x:v>
       </x:c>
-      <x:c r="B112" s="1" t="s">
+      <x:c r="O112" s="1" t="s">
         <x:v>4612</x:v>
-      </x:c>
-      <x:c r="O112" s="1" t="s">
-        <x:v>4613</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="60" customHeight="1">
       <x:c r="A113" s="1" t="s">
+        <x:v>4613</x:v>
+      </x:c>
+      <x:c r="B113" s="1" t="s">
         <x:v>4614</x:v>
       </x:c>
-      <x:c r="B113" s="1" t="s">
+      <x:c r="O113" s="1" t="s">
         <x:v>4615</x:v>
-      </x:c>
-      <x:c r="O113" s="1" t="s">
-        <x:v>4616</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="60" customHeight="1">
       <x:c r="A114" s="1" t="s">
+        <x:v>4616</x:v>
+      </x:c>
+      <x:c r="B114" s="1" t="s">
         <x:v>4617</x:v>
       </x:c>
-      <x:c r="B114" s="1" t="s">
+      <x:c r="O114" s="1" t="s">
         <x:v>4618</x:v>
-      </x:c>
-      <x:c r="O114" s="1" t="s">
-        <x:v>4619</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="60" customHeight="1">
       <x:c r="A115" s="1" t="s">
+        <x:v>4619</x:v>
+      </x:c>
+      <x:c r="B115" s="1" t="s">
         <x:v>4620</x:v>
       </x:c>
-      <x:c r="B115" s="1" t="s">
+      <x:c r="O115" s="1" t="s">
         <x:v>4621</x:v>
-      </x:c>
-      <x:c r="O115" s="1" t="s">
-        <x:v>4622</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="60" customHeight="1">
       <x:c r="A116" s="1" t="s">
+        <x:v>4622</x:v>
+      </x:c>
+      <x:c r="B116" s="1" t="s">
+        <x:v>4620</x:v>
+      </x:c>
+      <x:c r="O116" s="1" t="s">
         <x:v>4623</x:v>
-      </x:c>
-      <x:c r="B116" s="1" t="s">
-        <x:v>4621</x:v>
-      </x:c>
-      <x:c r="O116" s="1" t="s">
-        <x:v>4624</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="60" customHeight="1">
       <x:c r="A117" s="1" t="s">
+        <x:v>4624</x:v>
+      </x:c>
+      <x:c r="B117" s="1" t="s">
         <x:v>4625</x:v>
       </x:c>
-      <x:c r="B117" s="1" t="s">
+      <x:c r="O117" s="1" t="s">
         <x:v>4626</x:v>
-      </x:c>
-      <x:c r="O117" s="1" t="s">
-        <x:v>4627</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="60" customHeight="1">
       <x:c r="A118" s="1" t="s">
+        <x:v>4627</x:v>
+      </x:c>
+      <x:c r="B118" s="1" t="s">
         <x:v>4628</x:v>
       </x:c>
-      <x:c r="B118" s="1" t="s">
+      <x:c r="O118" s="1" t="s">
         <x:v>4629</x:v>
-      </x:c>
-      <x:c r="O118" s="1" t="s">
-        <x:v>4630</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="60" customHeight="1">
       <x:c r="A119" s="1" t="s">
+        <x:v>4630</x:v>
+      </x:c>
+      <x:c r="B119" s="1" t="s">
         <x:v>4631</x:v>
       </x:c>
-      <x:c r="B119" s="1" t="s">
+      <x:c r="O119" s="1" t="s">
         <x:v>4632</x:v>
-      </x:c>
-      <x:c r="O119" s="1" t="s">
-        <x:v>4633</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="60" customHeight="1">
       <x:c r="A120" s="1" t="s">
+        <x:v>4633</x:v>
+      </x:c>
+      <x:c r="B120" s="1" t="s">
         <x:v>4634</x:v>
       </x:c>
-      <x:c r="B120" s="1" t="s">
+      <x:c r="O120" s="1" t="s">
         <x:v>4635</x:v>
-      </x:c>
-      <x:c r="O120" s="1" t="s">
-        <x:v>4636</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="60" customHeight="1">
       <x:c r="A121" s="1" t="s">
+        <x:v>4636</x:v>
+      </x:c>
+      <x:c r="B121" s="1" t="s">
         <x:v>4637</x:v>
       </x:c>
-      <x:c r="B121" s="1" t="s">
+      <x:c r="O121" s="1" t="s">
         <x:v>4638</x:v>
-      </x:c>
-      <x:c r="O121" s="1" t="s">
-        <x:v>4639</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="60" customHeight="1">
       <x:c r="A122" s="1" t="s">
+        <x:v>4639</x:v>
+      </x:c>
+      <x:c r="B122" s="1" t="s">
         <x:v>4640</x:v>
       </x:c>
-      <x:c r="B122" s="1" t="s">
+      <x:c r="O122" s="1" t="s">
         <x:v>4641</x:v>
-      </x:c>
-      <x:c r="O122" s="1" t="s">
-        <x:v>4642</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="60" customHeight="1">
       <x:c r="A123" s="1" t="s">
+        <x:v>4642</x:v>
+      </x:c>
+      <x:c r="B123" s="1" t="s">
         <x:v>4643</x:v>
       </x:c>
-      <x:c r="B123" s="1" t="s">
+      <x:c r="O123" s="1" t="s">
         <x:v>4644</x:v>
-      </x:c>
-      <x:c r="O123" s="1" t="s">
-        <x:v>4645</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="60" customHeight="1">
       <x:c r="A124" s="4" t="s">
+        <x:v>4645</x:v>
+      </x:c>
+      <x:c r="O124" s="1" t="s">
         <x:v>4646</x:v>
-      </x:c>
-      <x:c r="O124" s="1" t="s">
-        <x:v>4647</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="60" customHeight="1">
       <x:c r="A126" s="1" t="s">
-        <x:v>4648</x:v>
+        <x:v>4647</x:v>
       </x:c>
       <x:c r="B126" s="15" t="s">
         <x:v>2145</x:v>
       </x:c>
       <x:c r="O126" s="1" t="s">
-        <x:v>4649</x:v>
-      </x:c>
+        <x:v>4648</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="str">
+        <x:v>ImitatorFullDesc</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>The Imitator can select a dead crewmate during a meeting and borrow their role for the next action round. The copied role starts with fresh resources and is restored to Imitator at the next meeting.</x:v>
+      </x:c>
+      <x:c r="C127"/>
+      <x:c r="D127"/>
+      <x:c r="E127"/>
+      <x:c r="F127"/>
+      <x:c r="G127"/>
+      <x:c r="H127"/>
+      <x:c r="I127"/>
+      <x:c r="J127"/>
+      <x:c r="K127"/>
+      <x:c r="L127"/>
+      <x:c r="M127"/>
+      <x:c r="N127"/>
+      <x:c r="O127" t="str">
+        <x:v>效颦者可在会议中选择一名死亡船员，并在下一个行动轮借用其职业。复制的职业以全新资源开始，并在下一次会议时恢复为效颦者。</x:v>
+      </x:c>
+      <x:c r="P127"/>
+      <x:c r="Q127"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" t="str">
+        <x:v>TrapperPlusFullDesc</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>The Trapper places hidden information traps. Players who remain inside long enough are recorded once per round. At the next meeting, the Trapper receives a shuffled anonymous list of their roles if enough players were recorded.</x:v>
+      </x:c>
+      <x:c r="C128"/>
+      <x:c r="D128"/>
+      <x:c r="E128"/>
+      <x:c r="F128"/>
+      <x:c r="G128"/>
+      <x:c r="H128"/>
+      <x:c r="I128"/>
+      <x:c r="J128"/>
+      <x:c r="K128"/>
+      <x:c r="L128"/>
+      <x:c r="M128"/>
+      <x:c r="N128"/>
+      <x:c r="O128" t="str">
+        <x:v>陷阱师可放置隐藏的信息陷阱。玩家在范围内停留足够久后，每轮会被记录一次。若记录人数达到要求，下一次会议将收到随机排序且不含身份的职业列表。</x:v>
+      </x:c>
+      <x:c r="P128"/>
+      <x:c r="Q128"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="str">
+        <x:v>AurialFullDesc</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>The Aurial has poor vision but can radiate all nearby players. After a player is hit enough times, their current faction is shown by name color: green crew, gray neutral, or red impostor. Exact roles are never revealed.</x:v>
+      </x:c>
+      <x:c r="C129"/>
+      <x:c r="D129"/>
+      <x:c r="E129"/>
+      <x:c r="F129"/>
+      <x:c r="G129"/>
+      <x:c r="H129"/>
+      <x:c r="I129"/>
+      <x:c r="J129"/>
+      <x:c r="K129"/>
+      <x:c r="L129"/>
+      <x:c r="M129"/>
+      <x:c r="N129"/>
+      <x:c r="O129" t="str">
+        <x:v>灵光师视野较差，但可辐射附近所有玩家。玩家累计被命中足够次数后，其当前阵营会以姓名颜色显示：绿色船员、灰色中立、红色内鬼；不会显示具体职业。</x:v>
+      </x:c>
+      <x:c r="P129"/>
+      <x:c r="Q129"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Normalize Aurial anonymous silhouettes
</commit_message>
<xml_diff>
--- a/Strings.xlsx
+++ b/Strings.xlsx
@@ -31166,12 +31166,12 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>See others as anonymous silhouettes and radiate them repeatedly to reveal faction colors.</t>
+          <t>See everyone as identical anonymous silhouettes and radiate them repeatedly to reveal faction colors.</t>
         </is>
       </c>
       <c r="O494" t="inlineStr">
         <is>
-          <t>??????????????????????</t>
+          <t>????????????????????????????</t>
         </is>
       </c>
     </row>
@@ -33915,12 +33915,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>The Aurial has poor vision and sees other players only as anonymous black silhouettes, without names or cosmetics. Radiate nearby players repeatedly; after enough hits, their entire silhouette changes to their current faction color: green crew, gray neutral, or red impostor. Exact roles are never revealed.</t>
+          <t>The Aurial has poor vision and sees every other player as the same standard-sized anonymous black silhouette, without names, cosmetics, or distinctive body shapes. Radiate nearby players repeatedly; after enough hits, their entire silhouette changes to their current faction color: green crew, gray neutral, or red impostor. Exact roles are never revealed.</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>???????????????????????????????????????????????????????????????????????????????????????</t>
+          <t>????????????????????????????????????????????????????????????????????????????????????????????????????</t>
         </is>
       </c>
     </row>

</xml_diff>